<commit_message>
Update Raboushee complete September & October attendance records
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I133"/>
+  <dimension ref="A1:I143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -810,12 +810,12 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Paid Standby</t>
+          <t>Paid Mission</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
+          <t>🏢 Official Airport Mission / Pass Delay (Company Paid)</t>
         </is>
       </c>
     </row>
@@ -1225,47 +1225,47 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Raboushee</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Rest Day (Contractual 1 Day Off in 7-day cycle)</t>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Paid Mission</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>🏢 Official Airport Mission / Pass Delay (Company Paid)</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1702,20 +1702,20 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Paid Mission</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Prep / Paid Administrative Standby (8h)</t>
+          <t>🏢 Official Airport Mission / Pass Delay (Company Paid)</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2197,20 +2197,20 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>8h 15m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>8.25</v>
+        <v>9</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Paid Shift</t>
+          <t>Paid Mission</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>🏢 Airport Onboarding Shift / Logged in 07:45 AM (8h 15m)</t>
+          <t>🏢 Official Airport Mission / Pass Delay (Company Paid)</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2705,7 @@
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Paid Standby</t>
         </is>
       </c>
     </row>
@@ -3182,16 +3182,16 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>04:05 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G60" s="4" t="n">
-        <v>8.08</v>
+        <v>8</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -3200,7 +3200,7 @@
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Paid Standby</t>
         </is>
       </c>
     </row>
@@ -3672,21 +3672,21 @@
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>7h 25m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G71" s="7" t="n">
-        <v>7.42</v>
+        <v>9.5</v>
       </c>
       <c r="H71" s="5" t="inlineStr">
         <is>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="I71" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
@@ -4167,21 +4167,21 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>07:50 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>7h 30m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G82" s="4" t="n">
-        <v>7.5</v>
+        <v>9.5</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -4190,7 +4190,7 @@
       </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:50 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
@@ -4662,7 +4662,7 @@
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>07:50 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -4672,20 +4672,20 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>12h 10m</t>
+          <t>13h 00m</t>
         </is>
       </c>
       <c r="G93" s="7" t="n">
-        <v>12.17</v>
+        <v>13</v>
       </c>
       <c r="H93" s="5" t="inlineStr">
         <is>
-          <t>Overtime</t>
+          <t>Extended Shift</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
         <is>
-          <t>✈️ Extended Duty (07:50 AM – 08:00 PM / 12h 05m) — ⚠️ Aircraft Technical Hazard: Fuel Leak Incident</t>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 08:00 PM / 13h 00m)</t>
         </is>
       </c>
     </row>
@@ -5157,30 +5157,30 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>03:15 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>12h 45m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G104" s="4" t="n">
-        <v>12.75</v>
+        <v>9.5</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I104" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Dawn Flight Departure Handling (Logged in 03:15 AM / Logged out 04:00 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
@@ -5675,7 +5675,7 @@
       </c>
       <c r="I115" s="9" t="inlineStr">
         <is>
-          <t>🌴 Scheduled Team Weekly Rest Day (Full Station Off)</t>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
@@ -5952,17 +5952,17 @@
     <row r="122" ht="20" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -5972,16 +5972,16 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G122" s="4" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
@@ -6007,7 +6007,7 @@
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D123" s="5" t="inlineStr">
@@ -6017,42 +6017,42 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F123" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G123" s="7" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H123" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I123" s="6" t="inlineStr">
         <is>
-          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="124" ht="20" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -6062,42 +6062,42 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>04:15 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>8h 15m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>8.25</v>
+        <v>8.5</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
         </is>
       </c>
     </row>
     <row r="125" ht="20" customHeight="1">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D125" s="5" t="inlineStr">
@@ -6120,24 +6120,24 @@
       </c>
       <c r="H125" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I125" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="126" ht="20" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -6152,16 +6152,16 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:15 PM</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 15m</t>
         </is>
       </c>
       <c r="G126" s="4" t="n">
-        <v>8</v>
+        <v>8.25</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -6177,12 +6177,12 @@
     <row r="127" ht="20" customHeight="1">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="D127" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
@@ -6202,11 +6202,11 @@
       </c>
       <c r="F127" s="5" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G127" s="7" t="n">
-        <v>8.08</v>
+        <v>8</v>
       </c>
       <c r="H127" s="5" t="inlineStr">
         <is>
@@ -6215,24 +6215,24 @@
       </c>
       <c r="I127" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="128" ht="20" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -6242,16 +6242,16 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -6267,12 +6267,12 @@
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="D129" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
@@ -6292,56 +6292,56 @@
       </c>
       <c r="F129" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G129" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H129" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I129" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="130" ht="20" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>07:55 AM</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>03:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 05m</t>
         </is>
       </c>
       <c r="G130" s="4" t="n">
-        <v>8.5</v>
+        <v>8.08</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -6350,64 +6350,64 @@
       </c>
       <c r="I130" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="131" ht="20" customHeight="1">
-      <c r="A131" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B131" s="8" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C131" s="9" t="inlineStr">
-        <is>
-          <t>Hanan</t>
-        </is>
-      </c>
-      <c r="D131" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E131" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F131" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G131" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H131" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I131" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F131" s="5" t="inlineStr">
+        <is>
+          <t>8h 00m</t>
+        </is>
+      </c>
+      <c r="G131" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H131" s="5" t="inlineStr">
+        <is>
+          <t>Training / Paid</t>
+        </is>
+      </c>
+      <c r="I131" s="6" t="inlineStr">
+        <is>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="132" ht="20" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -6417,75 +6417,525 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>03:15 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>13h 15m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G132" s="4" t="n">
-        <v>13.25</v>
+        <v>5.5</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I132" s="3" t="inlineStr">
         <is>
-          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="133" ht="20" customHeight="1">
       <c r="A133" s="5" t="inlineStr">
         <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>01:30 PM</t>
+        </is>
+      </c>
+      <c r="F133" s="5" t="inlineStr">
+        <is>
+          <t>5h 30m</t>
+        </is>
+      </c>
+      <c r="G133" s="7" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H133" s="5" t="inlineStr">
+        <is>
+          <t>Training / Paid</t>
+        </is>
+      </c>
+      <c r="I133" s="6" t="inlineStr">
+        <is>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="20" customHeight="1">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G134" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I134" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="20" customHeight="1">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F135" s="5" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G135" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H135" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I135" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="20" customHeight="1">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>03:30 PM</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>8h 30m</t>
+        </is>
+      </c>
+      <c r="G136" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I136" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="20" customHeight="1">
+      <c r="A137" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B137" s="8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C137" s="9" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E137" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F137" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G137" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I137" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="20" customHeight="1">
+      <c r="A138" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B138" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C138" s="9" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D138" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E138" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F138" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G138" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I138" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="20" customHeight="1">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C139" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F139" s="5" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G139" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H139" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I139" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="20" customHeight="1">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>03:15 AM</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>13h 15m</t>
+        </is>
+      </c>
+      <c r="G140" s="4" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>Dawn Shift</t>
+        </is>
+      </c>
+      <c r="I140" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="20" customHeight="1">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C141" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F141" s="5" t="inlineStr">
+        <is>
+          <t>9h 40m</t>
+        </is>
+      </c>
+      <c r="G141" s="7" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="H141" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I141" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="20" customHeight="1">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B133" s="5" t="inlineStr">
+      <c r="B142" s="2" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C133" s="6" t="inlineStr">
+      <c r="C142" s="3" t="inlineStr">
         <is>
           <t>Hanan</t>
         </is>
       </c>
-      <c r="D133" s="5" t="inlineStr">
+      <c r="D142" s="2" t="inlineStr">
         <is>
           <t>08:00 AM</t>
         </is>
       </c>
-      <c r="E133" s="5" t="inlineStr">
+      <c r="E142" s="2" t="inlineStr">
         <is>
           <t>05:00 PM</t>
         </is>
       </c>
-      <c r="F133" s="5" t="inlineStr">
+      <c r="F142" s="2" t="inlineStr">
         <is>
           <t>9h 00m</t>
         </is>
       </c>
-      <c r="G133" s="7" t="n">
+      <c r="G142" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="H133" s="5" t="inlineStr">
+      <c r="H142" s="2" t="inlineStr">
         <is>
           <t>Official Duty</t>
         </is>
       </c>
-      <c r="I133" s="6" t="inlineStr">
+      <c r="I142" s="3" t="inlineStr">
         <is>
           <t>✈️ Live Daily Ground Duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="20" customHeight="1">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>07:30 AM</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G143" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H143" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I143" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
@@ -8784,7 +9234,7 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>08:20 AM</t>
+          <t>08:10 AM</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -8794,11 +9244,11 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>7h 40m</t>
+          <t>7h 50m</t>
         </is>
       </c>
       <c r="G51" s="7" t="n">
-        <v>7.67</v>
+        <v>7.83</v>
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
@@ -8807,7 +9257,7 @@
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>Standard daytime shift (7h 40m)</t>
+          <t>Standard daytime shift (7h 50m)</t>
         </is>
       </c>
     </row>
@@ -8834,16 +9284,16 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>03:45 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>7h 30m</t>
+          <t>7h 45m</t>
         </is>
       </c>
       <c r="G52" s="4" t="n">
-        <v>7.5</v>
+        <v>7.75</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -8852,7 +9302,7 @@
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Standard daytime shift (7h 30m)</t>
+          <t>Standard daytime shift (7h 45m)</t>
         </is>
       </c>
     </row>
@@ -8919,7 +9369,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>07:15 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -8929,11 +9379,11 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>8h 45m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>8.75</v>
+        <v>9</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -8942,7 +9392,7 @@
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>Morning departure processing (8h 45m)</t>
+          <t>Morning departure processing (4:00 PM return)</t>
         </is>
       </c>
     </row>
@@ -8964,7 +9414,7 @@
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>07:20 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -8974,11 +9424,11 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>8h 40m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G55" s="7" t="n">
-        <v>8.67</v>
+        <v>9</v>
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
@@ -8987,7 +9437,7 @@
       </c>
       <c r="I55" s="6" t="inlineStr">
         <is>
-          <t>Morning departure processing (8h 40m)</t>
+          <t>Morning departure processing (4:00 PM return)</t>
         </is>
       </c>
     </row>
@@ -9009,7 +9459,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>07:20 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -9019,11 +9469,11 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>8h 40m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G56" s="4" t="n">
-        <v>8.67</v>
+        <v>9</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -9032,7 +9482,7 @@
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>Morning departure processing (8h 40m)</t>
+          <t>Morning departure processing (4:00 PM return)</t>
         </is>
       </c>
     </row>
@@ -9072,12 +9522,12 @@
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>Paid Standby</t>
+          <t>Paid Mission</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr">
         <is>
-          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
+          <t>🏢 Official Airport Mission / Pass Delay (Company Paid)</t>
         </is>
       </c>
     </row>
@@ -10243,20 +10693,20 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>66.67</v>
+        <v>69.33</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>107.09</v>
+        <v>169.67</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>173.76</v>
+        <v>239</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
@@ -10265,20 +10715,20 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>84.66</v>
+        <v>66.67</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>84.34999999999999</v>
+        <v>107.09</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>169.01</v>
+        <v>173.76</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -10287,17 +10737,17 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Mohamed Adnan</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>74.75</v>
+        <v>84.66</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>82.16</v>
+        <v>84.34999999999999</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>156.91</v>
+        <v>169.01</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>17</v>
@@ -10309,17 +10759,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>75</v>
+        <v>74.75</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>78</v>
+        <v>82.16</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>153</v>
+        <v>156.91</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>17</v>
@@ -10331,17 +10781,17 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>68.01000000000001</v>
+        <v>75</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>81.17</v>
+        <v>78</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>149.18</v>
+        <v>153</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>17</v>

</xml_diff>

<commit_message>
Update Rasheed Akel complete September & October attendance records
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I143"/>
+  <dimension ref="A1:I153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -837,30 +837,30 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>02:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>6h 15m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>🎓 Saudia Airlines Training Session (6h 15m) + Paid Standby</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -1270,47 +1270,47 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Rasheed Akel</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Rest Day (Contractual 1 Day Off in 7-day cycle)</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1747,20 +1747,20 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Prep / Paid Administrative Standby (8h)</t>
+          <t>✈️ Live Daily Ground Duty (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -2232,30 +2232,30 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G39" s="7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>Paid Standby</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -2727,7 +2727,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2737,20 +2737,20 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G50" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>✈️ Live Daily Ground Duty (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -3222,30 +3222,30 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>03:00 AM</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>04:05 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>13h 00m</t>
         </is>
       </c>
       <c r="G61" s="7" t="n">
-        <v>8.08</v>
+        <v>13</v>
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
         </is>
       </c>
     </row>
@@ -3717,21 +3717,21 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>03:55 AM</t>
+          <t>03:00 AM</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>11h 25m</t>
+          <t>13h 00m</t>
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>11.42</v>
+        <v>13</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3740,7 +3740,7 @@
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Dawn Flight Departure Handling (Logged in 03:55 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
         </is>
       </c>
     </row>
@@ -4212,21 +4212,21 @@
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>07:50 AM</t>
+          <t>03:00 AM</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>7h 30m</t>
+          <t>13h 00m</t>
         </is>
       </c>
       <c r="G83" s="7" t="n">
-        <v>7.5</v>
+        <v>13</v>
       </c>
       <c r="H83" s="5" t="inlineStr">
         <is>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:50 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
         </is>
       </c>
     </row>
@@ -4707,30 +4707,30 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>07:50 AM</t>
+          <t>03:00 AM</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>03:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>7h 40m</t>
+          <t>13h 00m</t>
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>7.67</v>
+        <v>13</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:50 AM / Logged out 03:30 PM)</t>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
         </is>
       </c>
     </row>
@@ -5202,21 +5202,21 @@
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>03:30 AM</t>
+          <t>03:00 AM</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>03:35 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>12h 05m</t>
+          <t>13h 00m</t>
         </is>
       </c>
       <c r="G105" s="7" t="n">
-        <v>12.08</v>
+        <v>13</v>
       </c>
       <c r="H105" s="5" t="inlineStr">
         <is>
@@ -5225,7 +5225,7 @@
       </c>
       <c r="I105" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Dawn Flight Departure Handling (Logged in 03:30 AM / Logged out 03:35 PM)</t>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
         </is>
       </c>
     </row>
@@ -5680,47 +5680,47 @@
       </c>
     </row>
     <row r="116" ht="20" customHeight="1">
-      <c r="A116" s="8" t="inlineStr">
+      <c r="A116" s="2" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="B116" s="8" t="inlineStr">
+      <c r="B116" s="2" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C116" s="9" t="inlineStr">
+      <c r="C116" s="3" t="inlineStr">
         <is>
           <t>Rasheed Akel</t>
         </is>
       </c>
-      <c r="D116" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E116" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F116" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G116" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H116" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I116" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Weekly Rest Day (Full Station Off)</t>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G116" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I116" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -5997,45 +5997,45 @@
     <row r="123" ht="20" customHeight="1">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D123" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F123" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G123" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H123" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I123" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6052,7 +6052,7 @@
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -6062,25 +6062,25 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
         <is>
-          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6097,7 @@
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D125" s="5" t="inlineStr">
@@ -6107,42 +6107,42 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F125" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G125" s="7" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H125" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I125" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
         </is>
       </c>
     </row>
     <row r="126" ht="20" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -6152,16 +6152,16 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>04:15 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>8h 15m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G126" s="4" t="n">
-        <v>8.25</v>
+        <v>8</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
@@ -6177,45 +6177,45 @@
     <row r="127" ht="20" customHeight="1">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D127" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F127" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G127" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H127" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I127" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6232,7 +6232,7 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -6242,16 +6242,16 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:15 PM</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 15m</t>
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>8</v>
+        <v>8.25</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
@@ -6267,17 +6267,17 @@
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D129" s="5" t="inlineStr">
@@ -6300,34 +6300,34 @@
       </c>
       <c r="H129" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I129" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="130" ht="20" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -6337,77 +6337,77 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G130" s="4" t="n">
-        <v>8.08</v>
+        <v>8</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I130" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="131" ht="20" customHeight="1">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B131" s="5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H131" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="132" ht="20" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -6422,16 +6422,16 @@
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G132" s="4" t="n">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -6447,67 +6447,67 @@
     <row r="133" ht="20" customHeight="1">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D133" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:55 AM</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F133" s="5" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>8h 05m</t>
         </is>
       </c>
       <c r="G133" s="7" t="n">
-        <v>5.5</v>
+        <v>8.08</v>
       </c>
       <c r="H133" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I133" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="134" ht="20" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -6517,77 +6517,77 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D135" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F135" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G135" s="7" t="n">
-        <v>9.5</v>
+        <v>6</v>
       </c>
       <c r="H135" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I135" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="136" ht="20" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -6597,137 +6597,137 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>01:30 PM</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>5h 30m</t>
+        </is>
+      </c>
+      <c r="G136" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>Training / Paid</t>
+        </is>
+      </c>
+      <c r="I136" s="3" t="inlineStr">
+        <is>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="20" customHeight="1">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C137" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>01:30 PM</t>
+        </is>
+      </c>
+      <c r="F137" s="5" t="inlineStr">
+        <is>
+          <t>5h 30m</t>
+        </is>
+      </c>
+      <c r="G137" s="7" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H137" s="5" t="inlineStr">
+        <is>
+          <t>Training / Paid</t>
+        </is>
+      </c>
+      <c r="I137" s="6" t="inlineStr">
+        <is>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="20" customHeight="1">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
           <t>07:00 AM</t>
         </is>
       </c>
-      <c r="E136" s="2" t="inlineStr">
-        <is>
-          <t>03:30 PM</t>
-        </is>
-      </c>
-      <c r="F136" s="2" t="inlineStr">
-        <is>
-          <t>8h 30m</t>
-        </is>
-      </c>
-      <c r="G136" s="4" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="H136" s="2" t="inlineStr">
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G138" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
         <is>
           <t>Official Duty</t>
         </is>
       </c>
-      <c r="I136" s="3" t="inlineStr">
-        <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
-        </is>
-      </c>
-    </row>
-    <row r="137" ht="20" customHeight="1">
-      <c r="A137" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B137" s="8" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C137" s="9" t="inlineStr">
-        <is>
-          <t>Raboushee</t>
-        </is>
-      </c>
-      <c r="D137" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E137" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F137" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G137" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H137" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I137" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
-        </is>
-      </c>
-    </row>
-    <row r="138" ht="20" customHeight="1">
-      <c r="A138" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B138" s="8" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C138" s="9" t="inlineStr">
-        <is>
-          <t>Hanan</t>
-        </is>
-      </c>
-      <c r="D138" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E138" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F138" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G138" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H138" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I138" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="I138" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="139" ht="20" customHeight="1">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D139" s="5" t="inlineStr">
@@ -6737,16 +6737,16 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F139" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G139" s="7" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="H139" s="5" t="inlineStr">
         <is>
@@ -6755,29 +6755,29 @@
       </c>
       <c r="I139" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>✈️ Live Morning Airport Ground Duty</t>
         </is>
       </c>
     </row>
     <row r="140" ht="20" customHeight="1">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>03:15 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
@@ -6787,155 +6787,605 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>13h 15m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>13.25</v>
+        <v>9.5</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
         <is>
-          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="141" ht="20" customHeight="1">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B141" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D141" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>03:00 AM</t>
         </is>
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t>04:40 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F141" s="5" t="inlineStr">
         <is>
-          <t>9h 40m</t>
+          <t>13h 00m</t>
         </is>
       </c>
       <c r="G141" s="7" t="n">
-        <v>9.67</v>
+        <v>13</v>
       </c>
       <c r="H141" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I141" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
         </is>
       </c>
     </row>
     <row r="142" ht="20" customHeight="1">
       <c r="A142" s="2" t="inlineStr">
         <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>03:30 PM</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>8h 30m</t>
+        </is>
+      </c>
+      <c r="G142" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I142" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="20" customHeight="1">
+      <c r="A143" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B143" s="8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C143" s="9" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D143" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E143" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F143" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G143" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I143" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>10h 30m</t>
+        </is>
+      </c>
+      <c r="G144" s="4" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I144" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:30 PM / 10h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="20" customHeight="1">
+      <c r="A145" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B145" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C145" s="9" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D145" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E145" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F145" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G145" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I145" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="20" customHeight="1">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G146" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I146" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="20" customHeight="1">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C147" s="6" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F147" s="5" t="inlineStr">
+        <is>
+          <t>5h 30m</t>
+        </is>
+      </c>
+      <c r="G147" s="7" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H147" s="5" t="inlineStr">
+        <is>
+          <t>Afternoon Duty</t>
+        </is>
+      </c>
+      <c r="I147" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Afternoon Station Duty (12:00 PM – 05:30 PM / 5h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="20" customHeight="1">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>03:15 AM</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>13h 15m</t>
+        </is>
+      </c>
+      <c r="G148" s="4" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>Dawn Shift</t>
+        </is>
+      </c>
+      <c r="I148" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="20" customHeight="1">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C149" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F149" s="5" t="inlineStr">
+        <is>
+          <t>9h 40m</t>
+        </is>
+      </c>
+      <c r="G149" s="7" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="H149" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I149" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="20" customHeight="1">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>05:40 PM</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>10h 40m</t>
+        </is>
+      </c>
+      <c r="G150" s="4" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I150" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="20" customHeight="1">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B142" s="2" t="inlineStr">
+      <c r="B151" s="5" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C142" s="3" t="inlineStr">
+      <c r="C151" s="6" t="inlineStr">
         <is>
           <t>Hanan</t>
         </is>
       </c>
-      <c r="D142" s="2" t="inlineStr">
+      <c r="D151" s="5" t="inlineStr">
         <is>
           <t>08:00 AM</t>
         </is>
       </c>
-      <c r="E142" s="2" t="inlineStr">
+      <c r="E151" s="5" t="inlineStr">
         <is>
           <t>05:00 PM</t>
         </is>
       </c>
-      <c r="F142" s="2" t="inlineStr">
+      <c r="F151" s="5" t="inlineStr">
         <is>
           <t>9h 00m</t>
         </is>
       </c>
-      <c r="G142" s="4" t="n">
+      <c r="G151" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="H142" s="2" t="inlineStr">
+      <c r="H151" s="5" t="inlineStr">
         <is>
           <t>Official Duty</t>
         </is>
       </c>
-      <c r="I142" s="3" t="inlineStr">
+      <c r="I151" s="6" t="inlineStr">
         <is>
           <t>✈️ Live Daily Ground Duty</t>
         </is>
       </c>
     </row>
-    <row r="143" ht="20" customHeight="1">
-      <c r="A143" s="5" t="inlineStr">
+    <row r="152" ht="20" customHeight="1">
+      <c r="A152" s="2" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B143" s="5" t="inlineStr">
+      <c r="B152" s="2" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C143" s="6" t="inlineStr">
+      <c r="C152" s="3" t="inlineStr">
         <is>
           <t>Raboushee</t>
         </is>
       </c>
-      <c r="D143" s="5" t="inlineStr">
+      <c r="D152" s="2" t="inlineStr">
         <is>
           <t>07:30 AM</t>
         </is>
       </c>
-      <c r="E143" s="5" t="inlineStr">
+      <c r="E152" s="2" t="inlineStr">
         <is>
           <t>05:00 PM</t>
         </is>
       </c>
-      <c r="F143" s="5" t="inlineStr">
+      <c r="F152" s="2" t="inlineStr">
         <is>
           <t>9h 30m</t>
         </is>
       </c>
-      <c r="G143" s="7" t="n">
+      <c r="G152" s="4" t="n">
         <v>9.5</v>
       </c>
-      <c r="H143" s="5" t="inlineStr">
+      <c r="H152" s="2" t="inlineStr">
         <is>
           <t>Official Duty</t>
         </is>
       </c>
-      <c r="I143" s="6" t="inlineStr">
+      <c r="I152" s="3" t="inlineStr">
         <is>
           <t>✈️ Live Daily Ground Duty (9h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="20" customHeight="1">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C153" s="6" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>10h 00m</t>
+        </is>
+      </c>
+      <c r="G153" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H153" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I153" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:00 PM / 10h 00m)</t>
         </is>
       </c>
     </row>
@@ -7749,30 +8199,30 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>06:30 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G18" s="4" t="n">
-        <v>9.5</v>
+        <v>8.5</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Standardized</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Standardized 23rd shift: 06:30 AM – 04:00 PM (9.5h)</t>
+          <t>Standard daytime shift (8h 30m)</t>
         </is>
       </c>
     </row>
@@ -7817,7 +8267,7 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Standard daytime shift</t>
+          <t>Standard daytime shift (8h 30m)</t>
         </is>
       </c>
     </row>
@@ -7844,16 +8294,16 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G20" s="4" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -7862,7 +8312,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Standard daytime shift</t>
+          <t>Standard daytime shift (8h 00m)</t>
         </is>
       </c>
     </row>
@@ -7889,16 +8339,16 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
@@ -7907,7 +8357,7 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Standard daytime shift</t>
+          <t>Standard daytime shift (8h 00m)</t>
         </is>
       </c>
     </row>
@@ -8064,7 +8514,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>03:00 AM</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -8074,20 +8524,20 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>13h 00m</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Paid Standby</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
         </is>
       </c>
     </row>
@@ -10671,20 +11121,20 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>75.08</v>
+        <v>77</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>177</v>
+        <v>196.17</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>252.08</v>
+        <v>273.17</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
@@ -10693,17 +11143,17 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>69.33</v>
+        <v>75.08</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>169.67</v>
+        <v>177</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>239</v>
+        <v>252.08</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>27</v>
@@ -10715,20 +11165,20 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>66.67</v>
+        <v>69.33</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>107.09</v>
+        <v>169.67</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>173.76</v>
+        <v>239</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -10737,20 +11187,20 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>84.66</v>
+        <v>66.67</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>84.34999999999999</v>
+        <v>107.09</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>169.01</v>
+        <v>173.76</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -10759,17 +11209,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Mohamed Adnan</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>74.75</v>
+        <v>84.66</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>82.16</v>
+        <v>84.34999999999999</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>156.91</v>
+        <v>169.01</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>17</v>
@@ -10781,17 +11231,17 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>75</v>
+        <v>74.75</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>78</v>
+        <v>82.16</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>153</v>
+        <v>156.91</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>17</v>

</xml_diff>

<commit_message>
Update Joudi Alghorani complete September & October attendance records
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I166"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1090,47 +1090,47 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Joudi Alghorani</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I14" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Rest Day (Contractual 1 Day Off in 7-day cycle)</t>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1612,20 +1612,20 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Paid Standby</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Prep / Paid Administrative Standby (8h)</t>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -2097,30 +2097,30 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>8h 15m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G36" s="4" t="n">
-        <v>8.25</v>
+        <v>9.5</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Paid Shift</t>
+          <t>Paid Standby</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>🏢 Airport Onboarding Shift / Logged in 07:45 AM (8h 15m)</t>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -2597,16 +2597,16 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G47" s="7" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Paid Standby</t>
         </is>
       </c>
     </row>
@@ -3092,16 +3092,16 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>04:05 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G58" s="4" t="n">
-        <v>8.08</v>
+        <v>8.5</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -3110,7 +3110,7 @@
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Paid Standby</t>
         </is>
       </c>
     </row>
@@ -3582,30 +3582,30 @@
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>7h 25m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G69" s="7" t="n">
-        <v>7.42</v>
+        <v>8</v>
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Dawn Flight Departure Handling (Logged in 07:55 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Daily Ground Duty (08:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -4077,30 +4077,30 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>04:45 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>10h 35m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G80" s="4" t="n">
-        <v>10.58</v>
+        <v>8</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Dawn Flight Departure Handling (Logged in 04:45 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Daily Ground Duty (08:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -4572,30 +4572,30 @@
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>04:45 AM</t>
+          <t>03:15 AM</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>03:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>10h 45m</t>
+          <t>12h 45m</t>
         </is>
       </c>
       <c r="G91" s="7" t="n">
-        <v>10.75</v>
+        <v>12.75</v>
       </c>
       <c r="H91" s="5" t="inlineStr">
         <is>
-          <t>Overtime</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 04:45 AM / Logged out 03:30 PM)</t>
+          <t>✈️ Early dawn flight departure handling (12h 45m)</t>
         </is>
       </c>
     </row>
@@ -5067,30 +5067,30 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>03:30 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>03:35 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>12h 05m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G102" s="4" t="n">
-        <v>12.08</v>
+        <v>9</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Dawn Flight Departure Handling (Logged in 03:30 AM / Logged out 03:35 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
         </is>
       </c>
     </row>
@@ -5545,47 +5545,47 @@
       </c>
     </row>
     <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="8" t="inlineStr">
+      <c r="A113" s="5" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="B113" s="8" t="inlineStr">
+      <c r="B113" s="5" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C113" s="9" t="inlineStr">
+      <c r="C113" s="6" t="inlineStr">
         <is>
           <t>Joudi Alghorani</t>
         </is>
       </c>
-      <c r="D113" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E113" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F113" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G113" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H113" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I113" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Weekly Rest Day (Full Station Off)</t>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G113" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="I113" s="6" t="inlineStr">
+        <is>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -6052,35 +6052,35 @@
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>08:20 AM</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>05:05 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>9h 05m</t>
+          <t>7h 40m</t>
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>9.08</v>
+        <v>7.67</v>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
         <is>
-          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 05:05 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6097,7 @@
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D125" s="5" t="inlineStr">
@@ -6107,25 +6107,25 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>05:05 PM</t>
         </is>
       </c>
       <c r="F125" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>9h 05m</t>
         </is>
       </c>
       <c r="G125" s="7" t="n">
-        <v>8.5</v>
+        <v>9.08</v>
       </c>
       <c r="H125" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I125" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 05:05 PM)</t>
         </is>
       </c>
     </row>
@@ -6142,7 +6142,7 @@
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -6187,80 +6187,80 @@
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D127" s="5" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F127" s="5" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G127" s="7" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="H127" s="5" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I127" s="6" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="128" ht="20" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6277,7 +6277,7 @@
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D129" s="5" t="inlineStr">
@@ -6287,25 +6287,25 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F129" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G129" s="7" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H129" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I129" s="6" t="inlineStr">
         <is>
-          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6322,26 +6322,26 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>08:05 AM</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>7h 55m</t>
         </is>
       </c>
       <c r="G130" s="4" t="n">
-        <v>8.5</v>
+        <v>7.92</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -6367,7 +6367,7 @@
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D131" s="5" t="inlineStr">
@@ -6377,25 +6377,25 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H131" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
         </is>
       </c>
     </row>
@@ -6412,52 +6412,52 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G132" s="4" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I132" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="133" ht="20" customHeight="1">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D133" s="5" t="inlineStr">
@@ -6467,16 +6467,16 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>04:15 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F133" s="5" t="inlineStr">
         <is>
-          <t>8h 15m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G133" s="7" t="n">
-        <v>8.25</v>
+        <v>8</v>
       </c>
       <c r="H133" s="5" t="inlineStr">
         <is>
@@ -6492,45 +6492,45 @@
     <row r="134" ht="20" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6547,7 +6547,7 @@
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D135" s="5" t="inlineStr">
@@ -6557,16 +6557,16 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:15 PM</t>
         </is>
       </c>
       <c r="F135" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 15m</t>
         </is>
       </c>
       <c r="G135" s="7" t="n">
-        <v>8.5</v>
+        <v>8.25</v>
       </c>
       <c r="H135" s="5" t="inlineStr">
         <is>
@@ -6592,7 +6592,7 @@
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -6637,52 +6637,52 @@
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D137" s="5" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F137" s="5" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G137" s="7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H137" s="5" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I137" s="6" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="138" ht="20" customHeight="1">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6692,16 +6692,16 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G138" s="4" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -6717,22 +6717,22 @@
     <row r="139" ht="20" customHeight="1">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D139" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E139" s="5" t="inlineStr">
@@ -6742,65 +6742,65 @@
       </c>
       <c r="F139" s="5" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G139" s="7" t="n">
-        <v>8.08</v>
+        <v>8</v>
       </c>
       <c r="H139" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I139" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="140" ht="20" customHeight="1">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6817,7 +6817,7 @@
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D141" s="5" t="inlineStr">
@@ -6862,92 +6862,92 @@
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="143" ht="20" customHeight="1">
       <c r="A143" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B143" s="5" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D143" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:55 AM</t>
         </is>
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F143" s="5" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>8h 05m</t>
         </is>
       </c>
       <c r="G143" s="7" t="n">
-        <v>5.5</v>
+        <v>8.08</v>
       </c>
       <c r="H143" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I143" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="144" ht="20" customHeight="1">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -6987,12 +6987,12 @@
     <row r="145" ht="20" customHeight="1">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B145" s="5" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C145" s="6" t="inlineStr">
@@ -7007,16 +7007,16 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F145" s="5" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G145" s="7" t="n">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="H145" s="5" t="inlineStr">
         <is>
@@ -7032,12 +7032,12 @@
     <row r="146" ht="20" customHeight="1">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
@@ -7047,42 +7047,42 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>9.5</v>
+        <v>6</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="147" ht="20" customHeight="1">
       <c r="A147" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B147" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C147" s="6" t="inlineStr">
@@ -7092,97 +7092,97 @@
       </c>
       <c r="D147" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F147" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G147" s="7" t="n">
-        <v>9</v>
+        <v>5.5</v>
       </c>
       <c r="H147" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I147" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="148" ht="20" customHeight="1">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>06:00 AM</t>
+          <t>08:10 AM</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>05:30 PM</t>
+          <t>01:00 PM</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>11h 30m</t>
+          <t>4h 50m</t>
         </is>
       </c>
       <c r="G148" s="4" t="n">
-        <v>11.5</v>
+        <v>4.83</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I148" s="3" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="149" ht="20" customHeight="1">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B149" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D149" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E149" s="5" t="inlineStr">
@@ -7192,82 +7192,82 @@
       </c>
       <c r="F149" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G149" s="7" t="n">
-        <v>9.5</v>
+        <v>8.5</v>
       </c>
       <c r="H149" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I149" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="150" ht="20" customHeight="1">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>03:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>13h 00m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G150" s="4" t="n">
-        <v>13</v>
+        <v>5.5</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I150" s="3" t="inlineStr">
         <is>
-          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="151" ht="20" customHeight="1">
       <c r="A151" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B151" s="5" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D151" s="5" t="inlineStr">
@@ -7277,16 +7277,16 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t>03:30 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F151" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G151" s="7" t="n">
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
       <c r="H151" s="5" t="inlineStr">
         <is>
@@ -7295,249 +7295,249 @@
       </c>
       <c r="I151" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="152" ht="20" customHeight="1">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>06:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>05:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>11h 30m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G152" s="4" t="n">
-        <v>11.5</v>
+        <v>9</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I152" s="3" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+          <t>✈️ Live Morning Airport Ground Duty</t>
         </is>
       </c>
     </row>
     <row r="153" ht="20" customHeight="1">
-      <c r="A153" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B153" s="8" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C153" s="9" t="inlineStr">
-        <is>
-          <t>Raboushee</t>
-        </is>
-      </c>
-      <c r="D153" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E153" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F153" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G153" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H153" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I153" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C153" s="6" t="inlineStr">
+        <is>
+          <t>Joudi Alghorani</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G153" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H153" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I153" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
         </is>
       </c>
     </row>
     <row r="154" ht="20" customHeight="1">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>06:00 AM</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G154" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I154" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="20" customHeight="1">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C155" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G155" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H155" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I155" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="20" customHeight="1">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
           <t>Rasheed Akel</t>
         </is>
       </c>
-      <c r="D154" s="2" t="inlineStr">
-        <is>
-          <t>07:00 AM</t>
-        </is>
-      </c>
-      <c r="E154" s="2" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F154" s="2" t="inlineStr">
-        <is>
-          <t>10h 30m</t>
-        </is>
-      </c>
-      <c r="G154" s="4" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H154" s="2" t="inlineStr">
-        <is>
-          <t>Extended Shift</t>
-        </is>
-      </c>
-      <c r="I154" s="3" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 05:30 PM / 10h 30m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="155" ht="20" customHeight="1">
-      <c r="A155" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B155" s="8" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C155" s="9" t="inlineStr">
-        <is>
-          <t>Hanan</t>
-        </is>
-      </c>
-      <c r="D155" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E155" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F155" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G155" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H155" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I155" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
-        </is>
-      </c>
-    </row>
-    <row r="156" ht="20" customHeight="1">
-      <c r="A156" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B156" s="8" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C156" s="9" t="inlineStr">
-        <is>
-          <t>Osama Alkabbani</t>
-        </is>
-      </c>
-      <c r="D156" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E156" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F156" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G156" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H156" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I156" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Contractual Paid Rest Day (Off Duty)</t>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>03:00 AM</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>13h 00m</t>
+        </is>
+      </c>
+      <c r="G156" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>Dawn Shift</t>
+        </is>
+      </c>
+      <c r="I156" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
         </is>
       </c>
     </row>
     <row r="157" ht="20" customHeight="1">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B157" s="5" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D157" s="5" t="inlineStr">
@@ -7547,16 +7547,16 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>03:30 PM</t>
         </is>
       </c>
       <c r="F157" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G157" s="7" t="n">
-        <v>9.5</v>
+        <v>8.5</v>
       </c>
       <c r="H157" s="5" t="inlineStr">
         <is>
@@ -7565,159 +7565,159 @@
       </c>
       <c r="I157" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>✈️ Live Morning Airport Ground Duty</t>
         </is>
       </c>
     </row>
     <row r="158" ht="20" customHeight="1">
-      <c r="A158" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B158" s="2" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C158" s="3" t="inlineStr">
-        <is>
-          <t>Rasheed Akel</t>
-        </is>
-      </c>
-      <c r="D158" s="2" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E158" s="2" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F158" s="2" t="inlineStr">
-        <is>
-          <t>5h 30m</t>
-        </is>
-      </c>
-      <c r="G158" s="4" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="H158" s="2" t="inlineStr">
-        <is>
-          <t>Afternoon Duty</t>
-        </is>
-      </c>
-      <c r="I158" s="3" t="inlineStr">
-        <is>
-          <t>✈️ Live Afternoon Station Duty (12:00 PM – 05:30 PM / 5h 30m)</t>
+      <c r="A158" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B158" s="8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C158" s="9" t="inlineStr">
+        <is>
+          <t>Joudi Alghorani</t>
+        </is>
+      </c>
+      <c r="D158" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E158" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F158" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G158" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I158" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="159" ht="20" customHeight="1">
       <c r="A159" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B159" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D159" s="5" t="inlineStr">
         <is>
-          <t>03:15 AM</t>
+          <t>06:00 AM</t>
         </is>
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>05:30 PM</t>
         </is>
       </c>
       <c r="F159" s="5" t="inlineStr">
         <is>
-          <t>13h 15m</t>
+          <t>11h 30m</t>
         </is>
       </c>
       <c r="G159" s="7" t="n">
-        <v>13.25</v>
+        <v>11.5</v>
       </c>
       <c r="H159" s="5" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Extended Shift</t>
         </is>
       </c>
       <c r="I159" s="6" t="inlineStr">
         <is>
-          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
         </is>
       </c>
     </row>
     <row r="160" ht="20" customHeight="1">
-      <c r="A160" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="B160" s="2" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C160" s="3" t="inlineStr">
-        <is>
-          <t>Osama Alkabbani</t>
-        </is>
-      </c>
-      <c r="D160" s="2" t="inlineStr">
-        <is>
-          <t>06:00 AM</t>
-        </is>
-      </c>
-      <c r="E160" s="2" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F160" s="2" t="inlineStr">
-        <is>
-          <t>11h 30m</t>
-        </is>
-      </c>
-      <c r="G160" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="H160" s="2" t="inlineStr">
-        <is>
-          <t>Extended Shift</t>
-        </is>
-      </c>
-      <c r="I160" s="3" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+      <c r="A160" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B160" s="8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C160" s="9" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D160" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E160" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F160" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G160" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I160" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="161" ht="20" customHeight="1">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B161" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D161" s="5" t="inlineStr">
@@ -7727,106 +7727,106 @@
       </c>
       <c r="E161" s="5" t="inlineStr">
         <is>
-          <t>04:40 PM</t>
+          <t>05:30 PM</t>
         </is>
       </c>
       <c r="F161" s="5" t="inlineStr">
         <is>
-          <t>9h 40m</t>
+          <t>10h 30m</t>
         </is>
       </c>
       <c r="G161" s="7" t="n">
-        <v>9.67</v>
+        <v>10.5</v>
       </c>
       <c r="H161" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Extended Shift</t>
         </is>
       </c>
       <c r="I161" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:30 PM / 10h 30m)</t>
         </is>
       </c>
     </row>
     <row r="162" ht="20" customHeight="1">
-      <c r="A162" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="B162" s="2" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C162" s="3" t="inlineStr">
-        <is>
-          <t>Rasheed Akel</t>
-        </is>
-      </c>
-      <c r="D162" s="2" t="inlineStr">
-        <is>
-          <t>07:00 AM</t>
-        </is>
-      </c>
-      <c r="E162" s="2" t="inlineStr">
-        <is>
-          <t>05:40 PM</t>
-        </is>
-      </c>
-      <c r="F162" s="2" t="inlineStr">
-        <is>
-          <t>10h 40m</t>
-        </is>
-      </c>
-      <c r="G162" s="4" t="n">
-        <v>10.67</v>
-      </c>
-      <c r="H162" s="2" t="inlineStr">
-        <is>
-          <t>Extended Shift</t>
-        </is>
-      </c>
-      <c r="I162" s="3" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+      <c r="A162" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B162" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D162" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E162" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F162" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G162" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I162" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="163" ht="20" customHeight="1">
       <c r="A163" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B163" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C163" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D163" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>05:00 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F163" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>8h 45m</t>
         </is>
       </c>
       <c r="G163" s="7" t="n">
-        <v>9</v>
+        <v>8.75</v>
       </c>
       <c r="H163" s="5" t="inlineStr">
         <is>
@@ -7835,64 +7835,64 @@
       </c>
       <c r="I163" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Ground Duty</t>
+          <t>✈️ Live Morning Airport Ground Duty (8h 45m)</t>
         </is>
       </c>
     </row>
     <row r="164" ht="20" customHeight="1">
-      <c r="A164" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="B164" s="2" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="C164" s="3" t="inlineStr">
+      <c r="A164" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B164" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C164" s="9" t="inlineStr">
         <is>
           <t>Osama Alkabbani</t>
         </is>
       </c>
-      <c r="D164" s="2" t="inlineStr">
-        <is>
-          <t>06:00 AM</t>
-        </is>
-      </c>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t>11h 30m</t>
-        </is>
-      </c>
-      <c r="G164" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="H164" s="2" t="inlineStr">
-        <is>
-          <t>Extended Shift</t>
-        </is>
-      </c>
-      <c r="I164" s="3" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+      <c r="D164" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E164" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F164" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G164" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I164" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Contractual Paid Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="165" ht="20" customHeight="1">
       <c r="A165" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B165" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C165" s="6" t="inlineStr">
@@ -7902,12 +7902,12 @@
       </c>
       <c r="D165" s="5" t="inlineStr">
         <is>
-          <t>07:30 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t>05:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F165" s="5" t="inlineStr">
@@ -7925,50 +7925,500 @@
       </c>
       <c r="I165" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Ground Duty (9h 30m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="166" ht="20" customHeight="1">
       <c r="A166" s="2" t="inlineStr">
         <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>5h 30m</t>
+        </is>
+      </c>
+      <c r="G166" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>Afternoon Duty</t>
+        </is>
+      </c>
+      <c r="I166" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Afternoon Station Duty (12:00 PM – 05:30 PM / 5h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="20" customHeight="1">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C167" s="6" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>03:15 AM</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F167" s="5" t="inlineStr">
+        <is>
+          <t>13h 15m</t>
+        </is>
+      </c>
+      <c r="G167" s="7" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="H167" s="5" t="inlineStr">
+        <is>
+          <t>Dawn Shift</t>
+        </is>
+      </c>
+      <c r="I167" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="20" customHeight="1">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>Joudi Alghorani</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>9h 20m</t>
+        </is>
+      </c>
+      <c r="G168" s="4" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I168" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 20m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="20" customHeight="1">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C169" s="6" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
+        <is>
+          <t>06:00 AM</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G169" s="7" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H169" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I169" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="20" customHeight="1">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>9h 40m</t>
+        </is>
+      </c>
+      <c r="G170" s="4" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I170" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="20" customHeight="1">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C171" s="6" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>05:40 PM</t>
+        </is>
+      </c>
+      <c r="F171" s="5" t="inlineStr">
+        <is>
+          <t>10h 40m</t>
+        </is>
+      </c>
+      <c r="G171" s="7" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="H171" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I171" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="20" customHeight="1">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B166" s="2" t="inlineStr">
+      <c r="B172" s="2" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C166" s="3" t="inlineStr">
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G172" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I172" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="20" customHeight="1">
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B173" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C173" s="6" t="inlineStr">
+        <is>
+          <t>Joudi Alghorani</t>
+        </is>
+      </c>
+      <c r="D173" s="5" t="inlineStr">
+        <is>
+          <t>07:30 AM</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="inlineStr">
+        <is>
+          <t>04:51 PM</t>
+        </is>
+      </c>
+      <c r="F173" s="5" t="inlineStr">
+        <is>
+          <t>9h 21m</t>
+        </is>
+      </c>
+      <c r="G173" s="7" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="H173" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I173" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (9h 21m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="20" customHeight="1">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>06:00 AM</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G174" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="20" customHeight="1">
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C175" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D175" s="5" t="inlineStr">
+        <is>
+          <t>07:30 AM</t>
+        </is>
+      </c>
+      <c r="E175" s="5" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F175" s="5" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G175" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H175" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I175" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (9h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="20" customHeight="1">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
         <is>
           <t>Rasheed Akel</t>
         </is>
       </c>
-      <c r="D166" s="2" t="inlineStr">
+      <c r="D176" s="2" t="inlineStr">
         <is>
           <t>07:00 AM</t>
         </is>
       </c>
-      <c r="E166" s="2" t="inlineStr">
+      <c r="E176" s="2" t="inlineStr">
         <is>
           <t>05:00 PM</t>
         </is>
       </c>
-      <c r="F166" s="2" t="inlineStr">
+      <c r="F176" s="2" t="inlineStr">
         <is>
           <t>10h 00m</t>
         </is>
       </c>
-      <c r="G166" s="4" t="n">
+      <c r="G176" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="H166" s="2" t="inlineStr">
+      <c r="H176" s="2" t="inlineStr">
         <is>
           <t>Extended Shift</t>
         </is>
       </c>
-      <c r="I166" s="3" t="inlineStr">
+      <c r="I176" s="3" t="inlineStr">
         <is>
           <t>⚡ Live Extended Station Duty (07:00 AM – 05:00 PM / 10h 00m)</t>
         </is>
@@ -12110,20 +12560,20 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>72</v>
+        <v>74.75</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>174</v>
+        <v>173.6</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>246</v>
+        <v>248.35</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -12132,17 +12582,17 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>69.33</v>
+        <v>72</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>169.67</v>
+        <v>174</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>27</v>
@@ -12154,20 +12604,20 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>66.67</v>
+        <v>69.33</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>107.09</v>
+        <v>169.67</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>173.76</v>
+        <v>239</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -12176,20 +12626,20 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>84.66</v>
+        <v>66.67</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>84.34999999999999</v>
+        <v>107.09</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>169.01</v>
+        <v>173.76</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -12198,17 +12648,17 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Mohamed Adnan</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>74.75</v>
+        <v>84.66</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>82.16</v>
+        <v>84.34999999999999</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>156.91</v>
+        <v>169.01</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>17</v>

</xml_diff>

<commit_message>
Update Khaled Malas complete October attendance records
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I176"/>
+  <dimension ref="A1:I186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -675,12 +675,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Paid Standby</t>
+          <t>Paid Mission</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
+          <t>🏢 Official Airport Mission / Pass Delay (Company Paid)</t>
         </is>
       </c>
     </row>
@@ -1135,47 +1135,47 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Khaled</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Rest Day (Contractual 1 Day Off in 7-day cycle)</t>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Paid Mission</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>🏢 Official Airport Mission / Pass Delay (Company Paid)</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1657,20 +1657,20 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G26" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Paid Mission</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Prep / Paid Administrative Standby (8h)</t>
+          <t>🏢 Official Airport Mission / Pass Delay (Company Paid)</t>
         </is>
       </c>
     </row>
@@ -2142,7 +2142,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2152,20 +2152,20 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>8h 15m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G37" s="7" t="n">
-        <v>8.25</v>
+        <v>9</v>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>Paid Shift</t>
+          <t>Paid Mission</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>🏢 Airport Onboarding Shift / Logged in 07:45 AM (8h 15m)</t>
+          <t>🏢 Official Airport Mission / Pass Delay (Company Paid)</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2647,11 +2647,11 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 15m</t>
         </is>
       </c>
       <c r="G48" s="4" t="n">
-        <v>8</v>
+        <v>8.25</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>🎓 Etihad IGS Training / HQ SERAVIA (07:45 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -3132,21 +3132,21 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:40 AM</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>04:05 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>8h 20m</t>
         </is>
       </c>
       <c r="G59" s="7" t="n">
-        <v>8.08</v>
+        <v>8.33</v>
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="I59" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>🎓 Etihad IGS Training / HQ SERAVIA (07:40 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -3627,21 +3627,21 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>07:13 AM</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>7h 25m</t>
+          <t>8h 47m</t>
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>7.42</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -3650,7 +3650,7 @@
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:13 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -4122,21 +4122,21 @@
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>07:50 AM</t>
+          <t>07:18 AM</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>7h 30m</t>
+          <t>8h 42m</t>
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>7.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H81" s="5" t="inlineStr">
         <is>
@@ -4145,7 +4145,7 @@
       </c>
       <c r="I81" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:50 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:18 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -4617,30 +4617,30 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>07:50 AM</t>
+          <t>07:05 AM</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>05:13 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>9h 23m</t>
+          <t>8h 55m</t>
         </is>
       </c>
       <c r="G92" s="4" t="n">
-        <v>9.380000000000001</v>
+        <v>8.92</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Overtime</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:50 AM / Logged out 05:13 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:05 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -5112,21 +5112,21 @@
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>07:47 AM</t>
+          <t>07:10 AM</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>03:35 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>7h 48m</t>
+          <t>8h 50m</t>
         </is>
       </c>
       <c r="G103" s="7" t="n">
-        <v>7.8</v>
+        <v>8.83</v>
       </c>
       <c r="H103" s="5" t="inlineStr">
         <is>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="I103" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:47 AM / Logged out 03:35 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:10 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -5590,47 +5590,47 @@
       </c>
     </row>
     <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="8" t="inlineStr">
+      <c r="A114" s="2" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="B114" s="8" t="inlineStr">
+      <c r="B114" s="2" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C114" s="9" t="inlineStr">
+      <c r="C114" s="3" t="inlineStr">
         <is>
           <t>Khaled</t>
         </is>
       </c>
-      <c r="D114" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E114" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F114" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G114" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H114" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I114" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Weekly Rest Day (Full Station Off)</t>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G114" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>Paid Mission</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>🏢 Official Airport Mission / Pass Delay (Company Paid)</t>
         </is>
       </c>
     </row>
@@ -6097,35 +6097,35 @@
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D125" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t>05:05 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F125" s="5" t="inlineStr">
         <is>
-          <t>9h 05m</t>
+          <t>8h 45m</t>
         </is>
       </c>
       <c r="G125" s="7" t="n">
-        <v>9.08</v>
+        <v>8.75</v>
       </c>
       <c r="H125" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I125" s="6" t="inlineStr">
         <is>
-          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 05:05 PM)</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:30 PM)</t>
         </is>
       </c>
     </row>
@@ -6142,7 +6142,7 @@
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -6152,25 +6152,25 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>05:05 PM</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>9h 05m</t>
         </is>
       </c>
       <c r="G126" s="4" t="n">
-        <v>8.5</v>
+        <v>9.08</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I126" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 05:05 PM)</t>
         </is>
       </c>
     </row>
@@ -6187,7 +6187,7 @@
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D127" s="5" t="inlineStr">
@@ -6232,80 +6232,80 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D129" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F129" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G129" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H129" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I129" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6322,12 +6322,12 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>08:05 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -6337,11 +6337,11 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>7h 55m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G130" s="4" t="n">
-        <v>7.92</v>
+        <v>8</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
@@ -6367,35 +6367,35 @@
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>08:05 AM</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>7h 55m</t>
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>8.5</v>
+        <v>7.92</v>
       </c>
       <c r="H131" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
         <is>
-          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6412,26 +6412,26 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:05 PM</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 20m</t>
         </is>
       </c>
       <c r="G132" s="4" t="n">
-        <v>8.5</v>
+        <v>8.33</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I132" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:05 PM)</t>
         </is>
       </c>
     </row>
@@ -6457,7 +6457,7 @@
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D133" s="5" t="inlineStr">
@@ -6467,25 +6467,25 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F133" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G133" s="7" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H133" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I133" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
         </is>
       </c>
     </row>
@@ -6502,52 +6502,52 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D135" s="5" t="inlineStr">
@@ -6557,16 +6557,16 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t>04:15 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F135" s="5" t="inlineStr">
         <is>
-          <t>8h 15m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G135" s="7" t="n">
-        <v>8.25</v>
+        <v>8</v>
       </c>
       <c r="H135" s="5" t="inlineStr">
         <is>
@@ -6582,45 +6582,45 @@
     <row r="136" ht="20" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G136" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I136" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D137" s="5" t="inlineStr">
@@ -6647,25 +6647,25 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:15 PM</t>
         </is>
       </c>
       <c r="F137" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 15m</t>
         </is>
       </c>
       <c r="G137" s="7" t="n">
-        <v>8</v>
+        <v>8.25</v>
       </c>
       <c r="H137" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I137" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -6692,16 +6692,16 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G138" s="4" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
@@ -6727,12 +6727,12 @@
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D139" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E139" s="5" t="inlineStr">
@@ -6742,11 +6742,11 @@
       </c>
       <c r="F139" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 15m</t>
         </is>
       </c>
       <c r="G139" s="7" t="n">
-        <v>8</v>
+        <v>8.25</v>
       </c>
       <c r="H139" s="5" t="inlineStr">
         <is>
@@ -6755,7 +6755,7 @@
       </c>
       <c r="I139" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6772,52 +6772,52 @@
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="141" ht="20" customHeight="1">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B141" s="5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D141" s="5" t="inlineStr">
@@ -6827,16 +6827,16 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F141" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G141" s="7" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H141" s="5" t="inlineStr">
         <is>
@@ -6852,17 +6852,17 @@
     <row r="142" ht="20" customHeight="1">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -6897,45 +6897,45 @@
     <row r="143" ht="20" customHeight="1">
       <c r="A143" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B143" s="5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D143" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F143" s="5" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G143" s="7" t="n">
-        <v>8.08</v>
+        <v>6</v>
       </c>
       <c r="H143" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I143" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6952,7 +6952,7 @@
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -6962,16 +6962,16 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G144" s="4" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -6997,7 +6997,7 @@
       </c>
       <c r="C145" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D145" s="5" t="inlineStr">
@@ -7042,116 +7042,116 @@
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>07:55 AM</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 05m</t>
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>6</v>
+        <v>8.08</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:55 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="147" ht="20" customHeight="1">
       <c r="A147" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B147" s="5" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C147" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D147" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:55 AM</t>
         </is>
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F147" s="5" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>8h 05m</t>
         </is>
       </c>
       <c r="G147" s="7" t="n">
-        <v>5.5</v>
+        <v>8.08</v>
       </c>
       <c r="H147" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I147" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="148" ht="20" customHeight="1">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>08:10 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>01:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>4h 50m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G148" s="4" t="n">
-        <v>4.83</v>
+        <v>8.5</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -7167,17 +7167,17 @@
     <row r="149" ht="20" customHeight="1">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B149" s="5" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D149" s="5" t="inlineStr">
@@ -7187,16 +7187,16 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F149" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G149" s="7" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H149" s="5" t="inlineStr">
         <is>
@@ -7212,45 +7212,45 @@
     <row r="150" ht="20" customHeight="1">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G150" s="4" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I150" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -7267,137 +7267,137 @@
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D151" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F151" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G151" s="7" t="n">
-        <v>9.5</v>
+        <v>5.5</v>
       </c>
       <c r="H151" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I151" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="152" ht="20" customHeight="1">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:10 AM</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>01:00 PM</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>4h 50m</t>
         </is>
       </c>
       <c r="G152" s="4" t="n">
-        <v>9</v>
+        <v>4.83</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I152" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="153" ht="20" customHeight="1">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D153" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F153" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>5h 45m</t>
         </is>
       </c>
       <c r="G153" s="7" t="n">
-        <v>9</v>
+        <v>5.75</v>
       </c>
       <c r="H153" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I153" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 01:30 PM)</t>
         </is>
       </c>
     </row>
     <row r="154" ht="20" customHeight="1">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
@@ -7407,42 +7407,42 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>06:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>05:30 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>11h 30m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>11.5</v>
+        <v>8.5</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="155" ht="20" customHeight="1">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B155" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C155" s="6" t="inlineStr">
@@ -7452,42 +7452,42 @@
       </c>
       <c r="D155" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E155" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F155" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G155" s="7" t="n">
-        <v>9.5</v>
+        <v>5.5</v>
       </c>
       <c r="H155" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I155" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="156" ht="20" customHeight="1">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C156" s="3" t="inlineStr">
@@ -7497,42 +7497,42 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>03:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>13h 00m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G156" s="4" t="n">
-        <v>13</v>
+        <v>9.5</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I156" s="3" t="inlineStr">
         <is>
-          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="157" ht="20" customHeight="1">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B157" s="5" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C157" s="6" t="inlineStr">
@@ -7547,16 +7547,16 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>03:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F157" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G157" s="7" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="H157" s="5" t="inlineStr">
         <is>
@@ -7570,263 +7570,263 @@
       </c>
     </row>
     <row r="158" ht="20" customHeight="1">
-      <c r="A158" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B158" s="8" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C158" s="9" t="inlineStr">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
         <is>
           <t>Joudi Alghorani</t>
         </is>
       </c>
-      <c r="D158" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E158" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F158" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G158" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H158" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I158" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G158" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I158" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
         </is>
       </c>
     </row>
     <row r="159" ht="20" customHeight="1">
       <c r="A159" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B159" s="5" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>07:10 AM</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>8h 50m</t>
+        </is>
+      </c>
+      <c r="G159" s="7" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="H159" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I159" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:10 AM – 04:00 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="20" customHeight="1">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
           <t>Osama Alkabbani</t>
         </is>
       </c>
-      <c r="D159" s="5" t="inlineStr">
+      <c r="D160" s="2" t="inlineStr">
         <is>
           <t>06:00 AM</t>
         </is>
       </c>
-      <c r="E159" s="5" t="inlineStr">
+      <c r="E160" s="2" t="inlineStr">
         <is>
           <t>05:30 PM</t>
         </is>
       </c>
-      <c r="F159" s="5" t="inlineStr">
+      <c r="F160" s="2" t="inlineStr">
         <is>
           <t>11h 30m</t>
         </is>
       </c>
-      <c r="G159" s="7" t="n">
+      <c r="G160" s="4" t="n">
         <v>11.5</v>
       </c>
-      <c r="H159" s="5" t="inlineStr">
+      <c r="H160" s="2" t="inlineStr">
         <is>
           <t>Extended Shift</t>
         </is>
       </c>
-      <c r="I159" s="6" t="inlineStr">
+      <c r="I160" s="3" t="inlineStr">
         <is>
           <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="160" ht="20" customHeight="1">
-      <c r="A160" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B160" s="8" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C160" s="9" t="inlineStr">
-        <is>
-          <t>Raboushee</t>
-        </is>
-      </c>
-      <c r="D160" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E160" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F160" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G160" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H160" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I160" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="161" ht="20" customHeight="1">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B161" s="5" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G161" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H161" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I161" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="20" customHeight="1">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
           <t>Rasheed Akel</t>
         </is>
       </c>
-      <c r="D161" s="5" t="inlineStr">
-        <is>
-          <t>07:00 AM</t>
-        </is>
-      </c>
-      <c r="E161" s="5" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F161" s="5" t="inlineStr">
-        <is>
-          <t>10h 30m</t>
-        </is>
-      </c>
-      <c r="G161" s="7" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H161" s="5" t="inlineStr">
-        <is>
-          <t>Extended Shift</t>
-        </is>
-      </c>
-      <c r="I161" s="6" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 05:30 PM / 10h 30m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="162" ht="20" customHeight="1">
-      <c r="A162" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B162" s="8" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>Hanan</t>
-        </is>
-      </c>
-      <c r="D162" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E162" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F162" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G162" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H162" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I162" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>03:00 AM</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>13h 00m</t>
+        </is>
+      </c>
+      <c r="G162" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>Dawn Shift</t>
+        </is>
+      </c>
+      <c r="I162" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
         </is>
       </c>
     </row>
     <row r="163" ht="20" customHeight="1">
       <c r="A163" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B163" s="5" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C163" s="6" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D163" s="5" t="inlineStr">
         <is>
-          <t>07:15 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:30 PM</t>
         </is>
       </c>
       <c r="F163" s="5" t="inlineStr">
         <is>
-          <t>8h 45m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G163" s="7" t="n">
-        <v>8.75</v>
+        <v>8.5</v>
       </c>
       <c r="H163" s="5" t="inlineStr">
         <is>
@@ -7835,24 +7835,24 @@
       </c>
       <c r="I163" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (8h 45m)</t>
+          <t>✈️ Live Morning Airport Ground Duty</t>
         </is>
       </c>
     </row>
     <row r="164" ht="20" customHeight="1">
       <c r="A164" s="8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B164" s="8" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C164" s="9" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D164" s="8" t="inlineStr">
@@ -7880,74 +7880,74 @@
       </c>
       <c r="I164" s="9" t="inlineStr">
         <is>
-          <t>🌴 Contractual Paid Rest Day (Off Duty)</t>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="165" ht="20" customHeight="1">
-      <c r="A165" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B165" s="5" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C165" s="6" t="inlineStr">
-        <is>
-          <t>Raboushee</t>
-        </is>
-      </c>
-      <c r="D165" s="5" t="inlineStr">
-        <is>
-          <t>07:00 AM</t>
-        </is>
-      </c>
-      <c r="E165" s="5" t="inlineStr">
-        <is>
-          <t>04:30 PM</t>
-        </is>
-      </c>
-      <c r="F165" s="5" t="inlineStr">
-        <is>
-          <t>9h 30m</t>
-        </is>
-      </c>
-      <c r="G165" s="7" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="H165" s="5" t="inlineStr">
-        <is>
-          <t>Official Duty</t>
-        </is>
-      </c>
-      <c r="I165" s="6" t="inlineStr">
-        <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+      <c r="A165" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B165" s="8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C165" s="9" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D165" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E165" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F165" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G165" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I165" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="166" ht="20" customHeight="1">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>06:00 AM</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
@@ -7957,191 +7957,191 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>11h 30m</t>
         </is>
       </c>
       <c r="G166" s="4" t="n">
-        <v>5.5</v>
+        <v>11.5</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>Afternoon Duty</t>
+          <t>Extended Shift</t>
         </is>
       </c>
       <c r="I166" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Afternoon Station Duty (12:00 PM – 05:30 PM / 5h 30m)</t>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
         </is>
       </c>
     </row>
     <row r="167" ht="20" customHeight="1">
-      <c r="A167" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="B167" s="5" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C167" s="6" t="inlineStr">
-        <is>
-          <t>Hanan</t>
-        </is>
-      </c>
-      <c r="D167" s="5" t="inlineStr">
-        <is>
-          <t>03:15 AM</t>
-        </is>
-      </c>
-      <c r="E167" s="5" t="inlineStr">
-        <is>
-          <t>04:30 PM</t>
-        </is>
-      </c>
-      <c r="F167" s="5" t="inlineStr">
-        <is>
-          <t>13h 15m</t>
-        </is>
-      </c>
-      <c r="G167" s="7" t="n">
-        <v>13.25</v>
-      </c>
-      <c r="H167" s="5" t="inlineStr">
-        <is>
-          <t>Dawn Shift</t>
-        </is>
-      </c>
-      <c r="I167" s="6" t="inlineStr">
-        <is>
-          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
+      <c r="A167" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B167" s="8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C167" s="9" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D167" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E167" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F167" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G167" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I167" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="168" ht="20" customHeight="1">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>07:20 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>04:40 PM</t>
+          <t>05:30 PM</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>9h 20m</t>
+          <t>10h 30m</t>
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>9.33</v>
+        <v>10.5</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Extended Shift</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 20m)</t>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:30 PM / 10h 30m)</t>
         </is>
       </c>
     </row>
     <row r="169" ht="20" customHeight="1">
-      <c r="A169" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="B169" s="5" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C169" s="6" t="inlineStr">
-        <is>
-          <t>Osama Alkabbani</t>
-        </is>
-      </c>
-      <c r="D169" s="5" t="inlineStr">
-        <is>
-          <t>06:00 AM</t>
-        </is>
-      </c>
-      <c r="E169" s="5" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F169" s="5" t="inlineStr">
-        <is>
-          <t>11h 30m</t>
-        </is>
-      </c>
-      <c r="G169" s="7" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="H169" s="5" t="inlineStr">
-        <is>
-          <t>Extended Shift</t>
-        </is>
-      </c>
-      <c r="I169" s="6" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+      <c r="A169" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B169" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C169" s="9" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D169" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E169" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F169" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G169" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I169" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="170" ht="20" customHeight="1">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>04:40 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>9h 40m</t>
+          <t>8h 45m</t>
         </is>
       </c>
       <c r="G170" s="4" t="n">
-        <v>9.67</v>
+        <v>8.75</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -8150,133 +8150,133 @@
       </c>
       <c r="I170" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (8h 45m)</t>
         </is>
       </c>
     </row>
     <row r="171" ht="20" customHeight="1">
       <c r="A171" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B171" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C171" s="6" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D171" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>07:07 AM</t>
         </is>
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t>05:40 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F171" s="5" t="inlineStr">
         <is>
-          <t>10h 40m</t>
+          <t>8h 53m</t>
         </is>
       </c>
       <c r="G171" s="7" t="n">
-        <v>10.67</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="H171" s="5" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I171" s="6" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:07 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="172" ht="20" customHeight="1">
-      <c r="A172" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="B172" s="2" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="C172" s="3" t="inlineStr">
-        <is>
-          <t>Hanan</t>
-        </is>
-      </c>
-      <c r="D172" s="2" t="inlineStr">
-        <is>
-          <t>08:00 AM</t>
-        </is>
-      </c>
-      <c r="E172" s="2" t="inlineStr">
-        <is>
-          <t>05:00 PM</t>
-        </is>
-      </c>
-      <c r="F172" s="2" t="inlineStr">
-        <is>
-          <t>9h 00m</t>
-        </is>
-      </c>
-      <c r="G172" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="H172" s="2" t="inlineStr">
-        <is>
-          <t>Official Duty</t>
-        </is>
-      </c>
-      <c r="I172" s="3" t="inlineStr">
-        <is>
-          <t>✈️ Live Daily Ground Duty</t>
+      <c r="A172" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B172" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C172" s="9" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D172" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E172" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F172" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G172" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I172" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Contractual Paid Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="173" ht="20" customHeight="1">
       <c r="A173" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B173" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C173" s="6" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D173" s="5" t="inlineStr">
         <is>
-          <t>07:30 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t>04:51 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F173" s="5" t="inlineStr">
         <is>
-          <t>9h 21m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G173" s="7" t="n">
-        <v>9.35</v>
+        <v>9.5</v>
       </c>
       <c r="H173" s="5" t="inlineStr">
         <is>
@@ -8285,29 +8285,29 @@
       </c>
       <c r="I173" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Ground Duty (9h 21m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="174" ht="20" customHeight="1">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>06:00 AM</t>
+          <t>12:00 PM</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
@@ -8317,108 +8317,558 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>11h 30m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G174" s="4" t="n">
-        <v>11.5</v>
+        <v>5.5</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Afternoon Duty</t>
         </is>
       </c>
       <c r="I174" s="3" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+          <t>✈️ Live Afternoon Station Duty (12:00 PM – 05:30 PM / 5h 30m)</t>
         </is>
       </c>
     </row>
     <row r="175" ht="20" customHeight="1">
       <c r="A175" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B175" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C175" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D175" s="5" t="inlineStr">
         <is>
-          <t>07:30 AM</t>
+          <t>03:15 AM</t>
         </is>
       </c>
       <c r="E175" s="5" t="inlineStr">
         <is>
-          <t>05:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F175" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>13h 15m</t>
         </is>
       </c>
       <c r="G175" s="7" t="n">
-        <v>9.5</v>
+        <v>13.25</v>
       </c>
       <c r="H175" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I175" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Ground Duty (9h 30m)</t>
+          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
         </is>
       </c>
     </row>
     <row r="176" ht="20" customHeight="1">
       <c r="A176" s="2" t="inlineStr">
         <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>Joudi Alghorani</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>9h 20m</t>
+        </is>
+      </c>
+      <c r="G176" s="4" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I176" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 20m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="20" customHeight="1">
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C177" s="6" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D177" s="5" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F177" s="5" t="inlineStr">
+        <is>
+          <t>9h 20m</t>
+        </is>
+      </c>
+      <c r="G177" s="7" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="H177" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I177" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 04:40 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="20" customHeight="1">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>06:00 AM</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G178" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I178" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="20" customHeight="1">
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C179" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D179" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E179" s="5" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F179" s="5" t="inlineStr">
+        <is>
+          <t>9h 40m</t>
+        </is>
+      </c>
+      <c r="G179" s="7" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="H179" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I179" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="20" customHeight="1">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>05:40 PM</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>10h 40m</t>
+        </is>
+      </c>
+      <c r="G180" s="4" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I180" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="20" customHeight="1">
+      <c r="A181" s="5" t="inlineStr">
+        <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B176" s="2" t="inlineStr">
+      <c r="B181" s="5" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C176" s="3" t="inlineStr">
+      <c r="C181" s="6" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D181" s="5" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F181" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G181" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H181" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I181" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="20" customHeight="1">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>Joudi Alghorani</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>07:30 AM</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>04:51 PM</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>9h 21m</t>
+        </is>
+      </c>
+      <c r="G182" s="4" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I182" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (9h 21m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="20" customHeight="1">
+      <c r="A183" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C183" s="6" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D183" s="5" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F183" s="5" t="inlineStr">
+        <is>
+          <t>9h 40m</t>
+        </is>
+      </c>
+      <c r="G183" s="7" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="H183" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I183" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 05:00 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="20" customHeight="1">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>06:00 AM</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G184" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I184" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="20" customHeight="1">
+      <c r="A185" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C185" s="6" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D185" s="5" t="inlineStr">
+        <is>
+          <t>07:30 AM</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F185" s="5" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G185" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H185" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I185" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (9h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="20" customHeight="1">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
         <is>
           <t>Rasheed Akel</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>07:00 AM</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>05:00 PM</t>
         </is>
       </c>
-      <c r="F176" s="2" t="inlineStr">
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>10h 00m</t>
         </is>
       </c>
-      <c r="G176" s="4" t="n">
+      <c r="G186" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="H176" s="2" t="inlineStr">
+      <c r="H186" s="2" t="inlineStr">
         <is>
           <t>Extended Shift</t>
         </is>
       </c>
-      <c r="I176" s="3" t="inlineStr">
+      <c r="I186" s="3" t="inlineStr">
         <is>
           <t>⚡ Live Extended Station Duty (07:00 AM – 05:00 PM / 10h 00m)</t>
         </is>
@@ -12604,20 +13054,20 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>69.33</v>
+        <v>71</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>169.67</v>
+        <v>172.68</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>239</v>
+        <v>243.68</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -12626,20 +13076,20 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>66.67</v>
+        <v>69.33</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>107.09</v>
+        <v>169.67</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>173.76</v>
+        <v>239</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -12648,20 +13098,20 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>84.66</v>
+        <v>66.67</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>84.34999999999999</v>
+        <v>107.09</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>169.01</v>
+        <v>173.76</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -12670,17 +13120,17 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Mohamed Adnan</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>71</v>
+        <v>84.66</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>73.42999999999999</v>
+        <v>84.34999999999999</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>144.43</v>
+        <v>169.01</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>17</v>

</xml_diff>

<commit_message>
Update Mohammad Almohammad (Mohamed Adnan) complete September & October records
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -488,12 +488,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I186"/>
+  <dimension ref="A1:I196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -697,7 +697,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1180,47 +1180,47 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Mohamed Adnan</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Rest Day (Contractual 1 Day Off in 7-day cycle)</t>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -1687,12 +1687,12 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1702,20 +1702,20 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Paid Standby</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Prep / Paid Administrative Standby (8h)</t>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Paid Standby</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -3182,16 +3182,16 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>04:05 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G60" s="4" t="n">
-        <v>8.08</v>
+        <v>8</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -3200,7 +3200,7 @@
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Paid Standby</t>
         </is>
       </c>
     </row>
@@ -3667,26 +3667,26 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>03:55 AM</t>
+          <t>08:40 AM</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>03:30 PM</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>11h 25m</t>
+          <t>6h 50m</t>
         </is>
       </c>
       <c r="G71" s="7" t="n">
-        <v>11.42</v>
+        <v>6.83</v>
       </c>
       <c r="H71" s="5" t="inlineStr">
         <is>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="I71" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 03:55 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (08:40 AM – 03:30 PM)</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -4172,25 +4172,25 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>03:30 PM</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>10h 35m</t>
+          <t>10h 45m</t>
         </is>
       </c>
       <c r="G82" s="4" t="n">
-        <v>10.58</v>
+        <v>10.75</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Dawn Flight Departure Handling (Logged in 04:45 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Early dawn flight departure handling (10h 45m)</t>
         </is>
       </c>
     </row>
@@ -4657,7 +4657,7 @@
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
@@ -4667,25 +4667,25 @@
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t>05:13 PM</t>
+          <t>05:00 PM</t>
         </is>
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>12h 28m</t>
+          <t>12h 15m</t>
         </is>
       </c>
       <c r="G93" s="7" t="n">
-        <v>12.47</v>
+        <v>12.25</v>
       </c>
       <c r="H93" s="5" t="inlineStr">
         <is>
-          <t>Overtime</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 04:45 AM / Logged out 05:13 PM)</t>
+          <t>✈️ Early dawn flight departure handling (12h 15m)</t>
         </is>
       </c>
     </row>
@@ -5152,26 +5152,26 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>07:47 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>03:35 PM</t>
+          <t>03:30 PM</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>7h 48m</t>
+          <t>7h 30m</t>
         </is>
       </c>
       <c r="G104" s="4" t="n">
-        <v>7.8</v>
+        <v>7.5</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="I104" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:47 AM / Logged out 03:35 PM)</t>
+          <t>✈️ Live Daily Ground Duty (08:00 AM – 03:30 PM)</t>
         </is>
       </c>
     </row>
@@ -5635,47 +5635,47 @@
       </c>
     </row>
     <row r="115" ht="20" customHeight="1">
-      <c r="A115" s="8" t="inlineStr">
+      <c r="A115" s="5" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="B115" s="8" t="inlineStr">
+      <c r="B115" s="5" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C115" s="9" t="inlineStr">
-        <is>
-          <t>Mohamed Adnan</t>
-        </is>
-      </c>
-      <c r="D115" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E115" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F115" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G115" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H115" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I115" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Weekly Rest Day (Full Station Off)</t>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G115" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H115" s="5" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="I115" s="6" t="inlineStr">
+        <is>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -6142,7 +6142,7 @@
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -6152,25 +6152,25 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>05:05 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>9h 05m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G126" s="4" t="n">
-        <v>9.08</v>
+        <v>8</v>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I126" s="3" t="inlineStr">
         <is>
-          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 05:05 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6187,7 +6187,7 @@
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D127" s="5" t="inlineStr">
@@ -6197,25 +6197,25 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>05:05 PM</t>
         </is>
       </c>
       <c r="F127" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>9h 05m</t>
         </is>
       </c>
       <c r="G127" s="7" t="n">
-        <v>8.5</v>
+        <v>9.08</v>
       </c>
       <c r="H127" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I127" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 05:05 PM)</t>
         </is>
       </c>
     </row>
@@ -6232,7 +6232,7 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -6277,80 +6277,80 @@
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D129" s="5" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F129" s="5" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G129" s="7" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="H129" s="5" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I129" s="6" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="130" ht="20" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G130" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I130" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6367,12 +6367,12 @@
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>08:05 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
@@ -6382,11 +6382,11 @@
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
-          <t>7h 55m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>7.92</v>
+        <v>8</v>
       </c>
       <c r="H131" s="5" t="inlineStr">
         <is>
@@ -6412,26 +6412,26 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>08:05 AM</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>04:05 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>8h 20m</t>
+          <t>7h 55m</t>
         </is>
       </c>
       <c r="G132" s="4" t="n">
-        <v>8.33</v>
+        <v>7.92</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I132" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:05 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6457,35 +6457,35 @@
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D133" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:05 PM</t>
         </is>
       </c>
       <c r="F133" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 20m</t>
         </is>
       </c>
       <c r="G133" s="7" t="n">
-        <v>8.5</v>
+        <v>8.33</v>
       </c>
       <c r="H133" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I133" s="6" t="inlineStr">
         <is>
-          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:05 PM)</t>
         </is>
       </c>
     </row>
@@ -6502,7 +6502,7 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -6512,16 +6512,16 @@
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
@@ -6547,7 +6547,7 @@
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D135" s="5" t="inlineStr">
@@ -6557,25 +6557,25 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F135" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G135" s="7" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H135" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I135" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
         </is>
       </c>
     </row>
@@ -6592,52 +6592,52 @@
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G136" s="4" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I136" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="137" ht="20" customHeight="1">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D137" s="5" t="inlineStr">
@@ -6647,16 +6647,16 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t>04:15 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F137" s="5" t="inlineStr">
         <is>
-          <t>8h 15m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G137" s="7" t="n">
-        <v>8.25</v>
+        <v>8</v>
       </c>
       <c r="H137" s="5" t="inlineStr">
         <is>
@@ -6672,45 +6672,45 @@
     <row r="138" ht="20" customHeight="1">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G138" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I138" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6727,17 +6727,17 @@
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D139" s="5" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:15 PM</t>
         </is>
       </c>
       <c r="F139" s="5" t="inlineStr">
@@ -6755,7 +6755,7 @@
       </c>
       <c r="I139" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -6795,12 +6795,12 @@
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6817,26 +6817,26 @@
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D141" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F141" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 15m</t>
         </is>
       </c>
       <c r="G141" s="7" t="n">
-        <v>8.5</v>
+        <v>8.25</v>
       </c>
       <c r="H141" s="5" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
       </c>
       <c r="I141" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6862,7 +6862,7 @@
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -6907,52 +6907,52 @@
       </c>
       <c r="C143" s="6" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D143" s="5" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F143" s="5" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G143" s="7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H143" s="5" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I143" s="6" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="144" ht="20" customHeight="1">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -6962,16 +6962,16 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G144" s="4" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -6987,17 +6987,17 @@
     <row r="145" ht="20" customHeight="1">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B145" s="5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C145" s="6" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D145" s="5" t="inlineStr">
@@ -7032,45 +7032,45 @@
     <row r="146" ht="20" customHeight="1">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>8.08</v>
+        <v>6</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:55 AM – 04:00 PM)</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -7087,12 +7087,12 @@
       </c>
       <c r="C147" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D147" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E147" s="5" t="inlineStr">
@@ -7102,20 +7102,20 @@
       </c>
       <c r="F147" s="5" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G147" s="7" t="n">
-        <v>8.08</v>
+        <v>8</v>
       </c>
       <c r="H147" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I147" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -7132,7 +7132,7 @@
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -7142,16 +7142,16 @@
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G148" s="4" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
@@ -7177,12 +7177,12 @@
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D149" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:55 AM</t>
         </is>
       </c>
       <c r="E149" s="5" t="inlineStr">
@@ -7192,11 +7192,11 @@
       </c>
       <c r="F149" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 05m</t>
         </is>
       </c>
       <c r="G149" s="7" t="n">
-        <v>8</v>
+        <v>8.08</v>
       </c>
       <c r="H149" s="5" t="inlineStr">
         <is>
@@ -7205,7 +7205,7 @@
       </c>
       <c r="I149" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:55 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -7222,116 +7222,116 @@
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G150" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I150" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="151" ht="20" customHeight="1">
       <c r="A151" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B151" s="5" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D151" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:55 AM</t>
         </is>
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F151" s="5" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>8h 05m</t>
         </is>
       </c>
       <c r="G151" s="7" t="n">
-        <v>5.5</v>
+        <v>8.08</v>
       </c>
       <c r="H151" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I151" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="152" ht="20" customHeight="1">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>08:10 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>01:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>4h 50m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G152" s="4" t="n">
-        <v>4.83</v>
+        <v>8.5</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -7347,36 +7347,36 @@
     <row r="153" ht="20" customHeight="1">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D153" s="5" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F153" s="5" t="inlineStr">
         <is>
-          <t>5h 45m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G153" s="7" t="n">
-        <v>5.75</v>
+        <v>8</v>
       </c>
       <c r="H153" s="5" t="inlineStr">
         <is>
@@ -7385,52 +7385,52 @@
       </c>
       <c r="I153" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 01:30 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="154" ht="20" customHeight="1">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -7447,7 +7447,7 @@
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D155" s="5" t="inlineStr">
@@ -7492,232 +7492,232 @@
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:10 AM</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>01:00 PM</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>4h 50m</t>
         </is>
       </c>
       <c r="G156" s="4" t="n">
-        <v>9.5</v>
+        <v>4.83</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I156" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="157" ht="20" customHeight="1">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B157" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D157" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F157" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>5h 45m</t>
         </is>
       </c>
       <c r="G157" s="7" t="n">
-        <v>9</v>
+        <v>5.75</v>
       </c>
       <c r="H157" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I157" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 01:30 PM)</t>
         </is>
       </c>
     </row>
     <row r="158" ht="20" customHeight="1">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>12:30 PM</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>4h 30m</t>
         </is>
       </c>
       <c r="G158" s="4" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I158" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="159" ht="20" customHeight="1">
       <c r="A159" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B159" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D159" s="5" t="inlineStr">
         <is>
-          <t>07:10 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F159" s="5" t="inlineStr">
         <is>
-          <t>8h 50m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G159" s="7" t="n">
-        <v>8.83</v>
+        <v>8.5</v>
       </c>
       <c r="H159" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I159" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (07:10 AM – 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="160" ht="20" customHeight="1">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>06:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>05:30 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>11h 30m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G160" s="4" t="n">
-        <v>11.5</v>
+        <v>5.5</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I160" s="3" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="161" ht="20" customHeight="1">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B161" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D161" s="5" t="inlineStr">
@@ -7762,12 +7762,12 @@
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>03:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
@@ -7777,37 +7777,37 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>13h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
         <is>
-          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
+          <t>✈️ Live Morning Airport Ground Duty</t>
         </is>
       </c>
     </row>
     <row r="163" ht="20" customHeight="1">
       <c r="A163" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B163" s="5" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C163" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D163" s="5" t="inlineStr">
@@ -7817,16 +7817,16 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>03:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F163" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G163" s="7" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="H163" s="5" t="inlineStr">
         <is>
@@ -7835,109 +7835,109 @@
       </c>
       <c r="I163" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
         </is>
       </c>
     </row>
     <row r="164" ht="20" customHeight="1">
-      <c r="A164" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B164" s="8" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C164" s="9" t="inlineStr">
-        <is>
-          <t>Joudi Alghorani</t>
-        </is>
-      </c>
-      <c r="D164" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E164" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F164" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G164" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H164" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I164" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>07:10 AM</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>8h 50m</t>
+        </is>
+      </c>
+      <c r="G164" s="4" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I164" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:10 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="165" ht="20" customHeight="1">
-      <c r="A165" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B165" s="8" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C165" s="9" t="inlineStr">
-        <is>
-          <t>Khaled</t>
-        </is>
-      </c>
-      <c r="D165" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E165" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F165" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G165" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H165" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I165" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C165" s="6" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F165" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G165" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H165" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I165" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
         </is>
       </c>
     </row>
     <row r="166" ht="20" customHeight="1">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -7975,488 +7975,488 @@
       </c>
     </row>
     <row r="167" ht="20" customHeight="1">
-      <c r="A167" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B167" s="8" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C167" s="9" t="inlineStr">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C167" s="6" t="inlineStr">
         <is>
           <t>Raboushee</t>
         </is>
       </c>
-      <c r="D167" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E167" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F167" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G167" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H167" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I167" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F167" s="5" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G167" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H167" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I167" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="168" ht="20" customHeight="1">
       <c r="A168" s="2" t="inlineStr">
         <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>03:00 AM</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>13h 00m</t>
+        </is>
+      </c>
+      <c r="G168" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>Dawn Shift</t>
+        </is>
+      </c>
+      <c r="I168" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="20" customHeight="1">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="B168" s="2" t="inlineStr">
+      <c r="B169" s="5" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C168" s="3" t="inlineStr">
-        <is>
-          <t>Rasheed Akel</t>
-        </is>
-      </c>
-      <c r="D168" s="2" t="inlineStr">
+      <c r="C169" s="6" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
         <is>
           <t>07:00 AM</t>
         </is>
       </c>
-      <c r="E168" s="2" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F168" s="2" t="inlineStr">
-        <is>
-          <t>10h 30m</t>
-        </is>
-      </c>
-      <c r="G168" s="4" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H168" s="2" t="inlineStr">
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>03:30 PM</t>
+        </is>
+      </c>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>8h 30m</t>
+        </is>
+      </c>
+      <c r="G169" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H169" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I169" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="20" customHeight="1">
+      <c r="A170" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B170" s="8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C170" s="9" t="inlineStr">
+        <is>
+          <t>Joudi Alghorani</t>
+        </is>
+      </c>
+      <c r="D170" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E170" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F170" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G170" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I170" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="20" customHeight="1">
+      <c r="A171" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B171" s="8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C171" s="9" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D171" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E171" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F171" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G171" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I171" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="20" customHeight="1">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>07:10 PM</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>12h 10m</t>
+        </is>
+      </c>
+      <c r="G172" s="4" t="n">
+        <v>12.17</v>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
         <is>
           <t>Extended Shift</t>
         </is>
       </c>
-      <c r="I168" s="3" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 05:30 PM / 10h 30m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="169" ht="20" customHeight="1">
-      <c r="A169" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B169" s="8" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C169" s="9" t="inlineStr">
-        <is>
-          <t>Hanan</t>
-        </is>
-      </c>
-      <c r="D169" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E169" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F169" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G169" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H169" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I169" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
-        </is>
-      </c>
-    </row>
-    <row r="170" ht="20" customHeight="1">
-      <c r="A170" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C170" s="3" t="inlineStr">
-        <is>
-          <t>Joudi Alghorani</t>
-        </is>
-      </c>
-      <c r="D170" s="2" t="inlineStr">
-        <is>
-          <t>07:15 AM</t>
-        </is>
-      </c>
-      <c r="E170" s="2" t="inlineStr">
-        <is>
-          <t>04:00 PM</t>
-        </is>
-      </c>
-      <c r="F170" s="2" t="inlineStr">
-        <is>
-          <t>8h 45m</t>
-        </is>
-      </c>
-      <c r="G170" s="4" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="H170" s="2" t="inlineStr">
-        <is>
-          <t>Official Duty</t>
-        </is>
-      </c>
-      <c r="I170" s="3" t="inlineStr">
-        <is>
-          <t>✈️ Live Morning Airport Ground Duty (8h 45m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="171" ht="20" customHeight="1">
-      <c r="A171" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B171" s="5" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C171" s="6" t="inlineStr">
-        <is>
-          <t>Khaled</t>
-        </is>
-      </c>
-      <c r="D171" s="5" t="inlineStr">
-        <is>
-          <t>07:07 AM</t>
-        </is>
-      </c>
-      <c r="E171" s="5" t="inlineStr">
-        <is>
-          <t>04:00 PM</t>
-        </is>
-      </c>
-      <c r="F171" s="5" t="inlineStr">
-        <is>
-          <t>8h 53m</t>
-        </is>
-      </c>
-      <c r="G171" s="7" t="n">
-        <v>8.880000000000001</v>
-      </c>
-      <c r="H171" s="5" t="inlineStr">
-        <is>
-          <t>Official Duty</t>
-        </is>
-      </c>
-      <c r="I171" s="6" t="inlineStr">
-        <is>
-          <t>✈️ Live Morning Airport Ground Duty (07:07 AM – 04:00 PM)</t>
-        </is>
-      </c>
-    </row>
-    <row r="172" ht="20" customHeight="1">
-      <c r="A172" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B172" s="8" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C172" s="9" t="inlineStr">
-        <is>
-          <t>Osama Alkabbani</t>
-        </is>
-      </c>
-      <c r="D172" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E172" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F172" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G172" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H172" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I172" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Contractual Paid Rest Day (Off Duty)</t>
+      <c r="I172" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 07:10 PM / 12h 10m)</t>
         </is>
       </c>
     </row>
     <row r="173" ht="20" customHeight="1">
       <c r="A173" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B173" s="5" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C173" s="6" t="inlineStr">
         <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D173" s="5" t="inlineStr">
+        <is>
+          <t>06:00 AM</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F173" s="5" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G173" s="7" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H173" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I173" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="20" customHeight="1">
+      <c r="A174" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B174" s="8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C174" s="9" t="inlineStr">
+        <is>
           <t>Raboushee</t>
         </is>
       </c>
-      <c r="D173" s="5" t="inlineStr">
-        <is>
-          <t>07:00 AM</t>
-        </is>
-      </c>
-      <c r="E173" s="5" t="inlineStr">
-        <is>
-          <t>04:30 PM</t>
-        </is>
-      </c>
-      <c r="F173" s="5" t="inlineStr">
-        <is>
-          <t>9h 30m</t>
-        </is>
-      </c>
-      <c r="G173" s="7" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="H173" s="5" t="inlineStr">
-        <is>
-          <t>Official Duty</t>
-        </is>
-      </c>
-      <c r="I173" s="6" t="inlineStr">
-        <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="174" ht="20" customHeight="1">
-      <c r="A174" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B174" s="2" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C174" s="3" t="inlineStr">
-        <is>
-          <t>Rasheed Akel</t>
-        </is>
-      </c>
-      <c r="D174" s="2" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E174" s="2" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F174" s="2" t="inlineStr">
-        <is>
-          <t>5h 30m</t>
-        </is>
-      </c>
-      <c r="G174" s="4" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="H174" s="2" t="inlineStr">
-        <is>
-          <t>Afternoon Duty</t>
-        </is>
-      </c>
-      <c r="I174" s="3" t="inlineStr">
-        <is>
-          <t>✈️ Live Afternoon Station Duty (12:00 PM – 05:30 PM / 5h 30m)</t>
+      <c r="D174" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E174" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F174" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G174" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H174" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I174" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="175" ht="20" customHeight="1">
       <c r="A175" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B175" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C175" s="6" t="inlineStr">
         <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D175" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E175" s="5" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F175" s="5" t="inlineStr">
+        <is>
+          <t>10h 30m</t>
+        </is>
+      </c>
+      <c r="G175" s="7" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H175" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I175" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:30 PM / 10h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="20" customHeight="1">
+      <c r="A176" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B176" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C176" s="9" t="inlineStr">
+        <is>
           <t>Hanan</t>
         </is>
       </c>
-      <c r="D175" s="5" t="inlineStr">
-        <is>
-          <t>03:15 AM</t>
-        </is>
-      </c>
-      <c r="E175" s="5" t="inlineStr">
-        <is>
-          <t>04:30 PM</t>
-        </is>
-      </c>
-      <c r="F175" s="5" t="inlineStr">
-        <is>
-          <t>13h 15m</t>
-        </is>
-      </c>
-      <c r="G175" s="7" t="n">
-        <v>13.25</v>
-      </c>
-      <c r="H175" s="5" t="inlineStr">
-        <is>
-          <t>Dawn Shift</t>
-        </is>
-      </c>
-      <c r="I175" s="6" t="inlineStr">
-        <is>
-          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="176" ht="20" customHeight="1">
-      <c r="A176" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C176" s="3" t="inlineStr">
-        <is>
-          <t>Joudi Alghorani</t>
-        </is>
-      </c>
-      <c r="D176" s="2" t="inlineStr">
-        <is>
-          <t>07:20 AM</t>
-        </is>
-      </c>
-      <c r="E176" s="2" t="inlineStr">
-        <is>
-          <t>04:40 PM</t>
-        </is>
-      </c>
-      <c r="F176" s="2" t="inlineStr">
-        <is>
-          <t>9h 20m</t>
-        </is>
-      </c>
-      <c r="G176" s="4" t="n">
-        <v>9.33</v>
-      </c>
-      <c r="H176" s="2" t="inlineStr">
-        <is>
-          <t>Official Duty</t>
-        </is>
-      </c>
-      <c r="I176" s="3" t="inlineStr">
-        <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 20m)</t>
+      <c r="D176" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E176" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F176" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G176" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I176" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="177" ht="20" customHeight="1">
       <c r="A177" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B177" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C177" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D177" s="5" t="inlineStr">
         <is>
-          <t>07:20 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E177" s="5" t="inlineStr">
         <is>
-          <t>04:40 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F177" s="5" t="inlineStr">
         <is>
-          <t>9h 20m</t>
+          <t>8h 45m</t>
         </is>
       </c>
       <c r="G177" s="7" t="n">
-        <v>9.33</v>
+        <v>8.75</v>
       </c>
       <c r="H177" s="5" t="inlineStr">
         <is>
@@ -8465,69 +8465,69 @@
       </c>
       <c r="I177" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 04:40 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (8h 45m)</t>
         </is>
       </c>
     </row>
     <row r="178" ht="20" customHeight="1">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>06:00 AM</t>
+          <t>07:07 AM</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>05:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>11h 30m</t>
+          <t>8h 53m</t>
         </is>
       </c>
       <c r="G178" s="4" t="n">
-        <v>11.5</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I178" s="3" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:07 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="179" ht="20" customHeight="1">
       <c r="A179" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B179" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D179" s="5" t="inlineStr">
@@ -8537,106 +8537,106 @@
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
-          <t>04:40 PM</t>
+          <t>06:30 PM</t>
         </is>
       </c>
       <c r="F179" s="5" t="inlineStr">
         <is>
-          <t>9h 40m</t>
+          <t>11h 30m</t>
         </is>
       </c>
       <c r="G179" s="7" t="n">
-        <v>9.67</v>
+        <v>11.5</v>
       </c>
       <c r="H179" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Extended Shift</t>
         </is>
       </c>
       <c r="I179" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 06:30 PM / 11h 30m)</t>
         </is>
       </c>
     </row>
     <row r="180" ht="20" customHeight="1">
-      <c r="A180" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="B180" s="2" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C180" s="3" t="inlineStr">
-        <is>
-          <t>Rasheed Akel</t>
-        </is>
-      </c>
-      <c r="D180" s="2" t="inlineStr">
-        <is>
-          <t>07:00 AM</t>
-        </is>
-      </c>
-      <c r="E180" s="2" t="inlineStr">
-        <is>
-          <t>05:40 PM</t>
-        </is>
-      </c>
-      <c r="F180" s="2" t="inlineStr">
-        <is>
-          <t>10h 40m</t>
-        </is>
-      </c>
-      <c r="G180" s="4" t="n">
-        <v>10.67</v>
-      </c>
-      <c r="H180" s="2" t="inlineStr">
-        <is>
-          <t>Extended Shift</t>
-        </is>
-      </c>
-      <c r="I180" s="3" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+      <c r="A180" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B180" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C180" s="9" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D180" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E180" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F180" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G180" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H180" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I180" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Contractual Paid Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="181" ht="20" customHeight="1">
       <c r="A181" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B181" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C181" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D181" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
-          <t>05:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F181" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G181" s="7" t="n">
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="H181" s="5" t="inlineStr">
         <is>
@@ -8645,230 +8645,680 @@
       </c>
       <c r="I181" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Ground Duty</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="182" ht="20" customHeight="1">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>07:30 AM</t>
+          <t>12:00 PM</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>04:51 PM</t>
+          <t>05:30 PM</t>
         </is>
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>9h 21m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G182" s="4" t="n">
-        <v>9.35</v>
+        <v>5.5</v>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Afternoon Duty</t>
         </is>
       </c>
       <c r="I182" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Ground Duty (9h 21m)</t>
+          <t>✈️ Live Afternoon Station Duty (12:00 PM – 05:30 PM / 5h 30m)</t>
         </is>
       </c>
     </row>
     <row r="183" ht="20" customHeight="1">
       <c r="A183" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B183" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C183" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D183" s="5" t="inlineStr">
         <is>
-          <t>07:20 AM</t>
+          <t>03:15 AM</t>
         </is>
       </c>
       <c r="E183" s="5" t="inlineStr">
         <is>
-          <t>05:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F183" s="5" t="inlineStr">
         <is>
-          <t>9h 40m</t>
+          <t>13h 15m</t>
         </is>
       </c>
       <c r="G183" s="7" t="n">
-        <v>9.67</v>
+        <v>13.25</v>
       </c>
       <c r="H183" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I183" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 05:00 PM)</t>
+          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
         </is>
       </c>
     </row>
     <row r="184" ht="20" customHeight="1">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>06:00 AM</t>
+          <t>07:20 AM</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>05:30 PM</t>
+          <t>04:40 PM</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>11h 30m</t>
+          <t>9h 20m</t>
         </is>
       </c>
       <c r="G184" s="4" t="n">
-        <v>11.5</v>
+        <v>9.33</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I184" s="3" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 20m)</t>
         </is>
       </c>
     </row>
     <row r="185" ht="20" customHeight="1">
       <c r="A185" s="5" t="inlineStr">
         <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C185" s="6" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D185" s="5" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F185" s="5" t="inlineStr">
+        <is>
+          <t>9h 20m</t>
+        </is>
+      </c>
+      <c r="G185" s="7" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="H185" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I185" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 04:40 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="20" customHeight="1">
+      <c r="A186" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B186" s="8" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C186" s="9" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D186" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E186" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F186" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G186" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H186" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I186" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="20" customHeight="1">
+      <c r="A187" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C187" s="6" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D187" s="5" t="inlineStr">
+        <is>
+          <t>06:00 AM</t>
+        </is>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F187" s="5" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G187" s="7" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H187" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I187" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="20" customHeight="1">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>9h 40m</t>
+        </is>
+      </c>
+      <c r="G188" s="4" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I188" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="20" customHeight="1">
+      <c r="A189" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C189" s="6" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D189" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>05:40 PM</t>
+        </is>
+      </c>
+      <c r="F189" s="5" t="inlineStr">
+        <is>
+          <t>10h 40m</t>
+        </is>
+      </c>
+      <c r="G189" s="7" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="H189" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I189" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="20" customHeight="1">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B185" s="5" t="inlineStr">
+      <c r="B190" s="2" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C185" s="6" t="inlineStr">
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G190" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I190" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="20" customHeight="1">
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C191" s="6" t="inlineStr">
+        <is>
+          <t>Joudi Alghorani</t>
+        </is>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>07:30 AM</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>04:51 PM</t>
+        </is>
+      </c>
+      <c r="F191" s="5" t="inlineStr">
+        <is>
+          <t>9h 21m</t>
+        </is>
+      </c>
+      <c r="G191" s="7" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="H191" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I191" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (9h 21m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="20" customHeight="1">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>9h 40m</t>
+        </is>
+      </c>
+      <c r="G192" s="4" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I192" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 05:00 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="20" customHeight="1">
+      <c r="A193" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C193" s="6" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>05:40 PM</t>
+        </is>
+      </c>
+      <c r="F193" s="5" t="inlineStr">
+        <is>
+          <t>10h 40m</t>
+        </is>
+      </c>
+      <c r="G193" s="7" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="H193" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I193" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="20" customHeight="1">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>06:00 AM</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G194" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I194" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="20" customHeight="1">
+      <c r="A195" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C195" s="6" t="inlineStr">
         <is>
           <t>Raboushee</t>
         </is>
       </c>
-      <c r="D185" s="5" t="inlineStr">
+      <c r="D195" s="5" t="inlineStr">
         <is>
           <t>07:30 AM</t>
         </is>
       </c>
-      <c r="E185" s="5" t="inlineStr">
+      <c r="E195" s="5" t="inlineStr">
         <is>
           <t>05:00 PM</t>
         </is>
       </c>
-      <c r="F185" s="5" t="inlineStr">
+      <c r="F195" s="5" t="inlineStr">
         <is>
           <t>9h 30m</t>
         </is>
       </c>
-      <c r="G185" s="7" t="n">
+      <c r="G195" s="7" t="n">
         <v>9.5</v>
       </c>
-      <c r="H185" s="5" t="inlineStr">
+      <c r="H195" s="5" t="inlineStr">
         <is>
           <t>Official Duty</t>
         </is>
       </c>
-      <c r="I185" s="6" t="inlineStr">
+      <c r="I195" s="6" t="inlineStr">
         <is>
           <t>✈️ Live Daily Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
-    <row r="186" ht="20" customHeight="1">
-      <c r="A186" s="2" t="inlineStr">
+    <row r="196" ht="20" customHeight="1">
+      <c r="A196" s="2" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="B196" s="2" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C186" s="3" t="inlineStr">
+      <c r="C196" s="3" t="inlineStr">
         <is>
           <t>Rasheed Akel</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D196" s="2" t="inlineStr">
         <is>
           <t>07:00 AM</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E196" s="2" t="inlineStr">
         <is>
           <t>05:00 PM</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
+      <c r="F196" s="2" t="inlineStr">
         <is>
           <t>10h 00m</t>
         </is>
       </c>
-      <c r="G186" s="4" t="n">
+      <c r="G196" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="H186" s="2" t="inlineStr">
+      <c r="H196" s="2" t="inlineStr">
         <is>
           <t>Extended Shift</t>
         </is>
       </c>
-      <c r="I186" s="3" t="inlineStr">
+      <c r="I196" s="3" t="inlineStr">
         <is>
           <t>⚡ Live Extended Station Duty (07:00 AM – 05:00 PM / 10h 00m)</t>
         </is>
@@ -8890,7 +9340,7 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -9094,35 +9544,35 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>06:30 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
-        <v>9.5</v>
+        <v>8.5</v>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Standardized</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Standardized 23rd shift: 06:30 AM – 04:00 PM (9.5h)</t>
+          <t>Standard daytime shift (8h 30m)</t>
         </is>
       </c>
     </row>
@@ -9589,7 +10039,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -9617,7 +10067,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Standard daytime shift</t>
+          <t>Standard daytime shift (8h 30m)</t>
         </is>
       </c>
     </row>
@@ -10084,7 +10534,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -10112,7 +10562,7 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Standard daytime shift</t>
+          <t>Standard daytime shift (8h 30m)</t>
         </is>
       </c>
     </row>
@@ -10579,7 +11029,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -10607,7 +11057,7 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>✈️ Dawn flight check-in &amp; boarding ops (12.83 hrs)</t>
+          <t>✈️ Early dawn flight departure handling (12h 50m)</t>
         </is>
       </c>
     </row>
@@ -11074,7 +11524,7 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
@@ -11084,16 +11534,16 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>12h 20m</t>
+          <t>12h 50m</t>
         </is>
       </c>
       <c r="G49" s="7" t="n">
-        <v>12.33</v>
+        <v>12.83</v>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
@@ -11102,7 +11552,7 @@
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>✈️ Dawn flight check-in &amp; boarding ops (12.33 hrs)</t>
+          <t>✈️ Early dawn flight departure handling (12h 50m)</t>
         </is>
       </c>
     </row>
@@ -11569,7 +12019,7 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -11579,16 +12029,16 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>12h 00m</t>
+          <t>12h 30m</t>
         </is>
       </c>
       <c r="G60" s="4" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -11597,7 +12047,7 @@
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>✈️ Early morning departure ops (12.0 hrs)</t>
+          <t>✈️ Early morning departure ops (12h 30m)</t>
         </is>
       </c>
     </row>
@@ -12064,7 +12514,7 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
@@ -12074,16 +12524,16 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>12h 00m</t>
+          <t>12h 30m</t>
         </is>
       </c>
       <c r="G71" s="7" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="H71" s="5" t="inlineStr">
         <is>
@@ -12092,7 +12542,7 @@
       </c>
       <c r="I71" s="6" t="inlineStr">
         <is>
-          <t>✈️ Early morning departure ops (12.0 hrs)</t>
+          <t>✈️ Early morning departure ops (12h 30m)</t>
         </is>
       </c>
     </row>
@@ -12559,7 +13009,7 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -12921,7 +13371,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -12988,20 +13438,20 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>75.08</v>
+        <v>85.16</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>177</v>
+        <v>178.17</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>252.08</v>
+        <v>263.3299999999999</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
@@ -13010,20 +13460,20 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>74.75</v>
+        <v>75.08</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>173.6</v>
+        <v>177</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>248.35</v>
+        <v>252.08</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -13032,20 +13482,20 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>72</v>
+        <v>74.75</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>174</v>
+        <v>173.6</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>246</v>
+        <v>248.35</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -13054,20 +13504,20 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>172.68</v>
+        <v>174</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>243.68</v>
+        <v>246</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -13076,20 +13526,20 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>69.33</v>
+        <v>71</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>169.67</v>
+        <v>172.68</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>239</v>
+        <v>243.68</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -13098,20 +13548,20 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>66.67</v>
+        <v>69.33</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>107.09</v>
+        <v>169.67</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>173.76</v>
+        <v>239</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -13120,20 +13570,20 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Mohamed Adnan</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>84.66</v>
+        <v>66.67</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>84.34999999999999</v>
+        <v>107.09</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>169.01</v>
+        <v>173.76</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Update Yasmin complete September & October attendance records
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I196"/>
+  <dimension ref="A1:I206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1022,25 +1022,25 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>02:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>6h 15m</t>
+          <t>7h 15m</t>
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>6.25</v>
+        <v>7.25</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>🎓 Saudia Airlines Training Session (6h 15m) + Paid Standby</t>
+          <t>🎓 Training Session (07:45 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -1495,47 +1495,47 @@
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Yasmin</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Rest Day (Contractual 1 Day Off in 7-day cycle)</t>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2017,20 +2017,20 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Paid Standby</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Prep / Paid Administrative Standby (8h)</t>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -2502,30 +2502,30 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>7h 00m</t>
         </is>
       </c>
       <c r="G45" s="7" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>Paid Standby</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
+          <t>🎓 Training Session (08:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -2997,7 +2997,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:30 AM</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -3007,20 +3007,20 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G56" s="4" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 1 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:30 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -3492,30 +3492,30 @@
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>04:05 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G67" s="7" t="n">
-        <v>8.08</v>
+        <v>9</v>
       </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad IGS Training Day 2 (MS Teams) / Saudi KSA Delegation / Paid Standby</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -3987,21 +3987,21 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>04:00 AM</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>7h 25m</t>
+          <t>12h 00m</t>
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>7.42</v>
+        <v>12</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Dawn Flight Departure Handling (Logged in 07:55 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Early dawn flight departure handling (12h 00m)</t>
         </is>
       </c>
     </row>
@@ -4482,30 +4482,30 @@
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>07:50 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>7h 30m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G89" s="7" t="n">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="H89" s="5" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:50 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -4977,21 +4977,21 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>07:50 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>03:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>7h 40m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G100" s="4" t="n">
-        <v>7.67</v>
+        <v>9</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="I100" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:50 AM / Logged out 03:30 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -5472,21 +5472,21 @@
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t>07:47 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>03:35 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>7h 48m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G111" s="7" t="n">
-        <v>7.8</v>
+        <v>9</v>
       </c>
       <c r="H111" s="5" t="inlineStr">
         <is>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="I111" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:47 AM / Logged out 03:35 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -5950,47 +5950,47 @@
       </c>
     </row>
     <row r="122" ht="20" customHeight="1">
-      <c r="A122" s="8" t="inlineStr">
+      <c r="A122" s="2" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="B122" s="8" t="inlineStr">
+      <c r="B122" s="2" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C122" s="9" t="inlineStr">
+      <c r="C122" s="3" t="inlineStr">
         <is>
           <t>Yasmin</t>
         </is>
       </c>
-      <c r="D122" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E122" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F122" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G122" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H122" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I122" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Weekly Rest Day (Full Station Off)</t>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="I122" s="3" t="inlineStr">
+        <is>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -6357,36 +6357,36 @@
     <row r="131" ht="20" customHeight="1">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B131" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Yasmin</t>
         </is>
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H131" s="5" t="inlineStr">
         <is>
@@ -6395,7 +6395,7 @@
       </c>
       <c r="I131" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>🎓 Training Session (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6412,12 +6412,12 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>08:05 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -6427,11 +6427,11 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>7h 55m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G132" s="4" t="n">
-        <v>7.92</v>
+        <v>8</v>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
@@ -6457,26 +6457,26 @@
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D133" s="5" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>08:05 AM</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>04:05 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F133" s="5" t="inlineStr">
         <is>
-          <t>8h 20m</t>
+          <t>7h 55m</t>
         </is>
       </c>
       <c r="G133" s="7" t="n">
-        <v>8.33</v>
+        <v>7.92</v>
       </c>
       <c r="H133" s="5" t="inlineStr">
         <is>
@@ -6485,7 +6485,7 @@
       </c>
       <c r="I133" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:05 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6502,26 +6502,26 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Mohammad Almohammad</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:05 PM</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 20m</t>
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>8</v>
+        <v>8.33</v>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="I134" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:05 PM)</t>
         </is>
       </c>
     </row>
@@ -6547,7 +6547,7 @@
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D135" s="5" t="inlineStr">
@@ -6557,25 +6557,25 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F135" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G135" s="7" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H135" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I135" s="6" t="inlineStr">
         <is>
-          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6592,7 +6592,7 @@
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -6615,12 +6615,12 @@
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I136" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Etihad DCS Systems Training &amp; Station Duty (Logged in 08:00 AM / Logged out 04:30 PM)</t>
         </is>
       </c>
     </row>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D137" s="5" t="inlineStr">
@@ -6647,16 +6647,16 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F137" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G137" s="7" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="H137" s="5" t="inlineStr">
         <is>
@@ -6682,116 +6682,116 @@
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G138" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I138" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="139" ht="20" customHeight="1">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D139" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t>04:15 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F139" s="5" t="inlineStr">
         <is>
-          <t>8h 15m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G139" s="7" t="n">
-        <v>8.25</v>
+        <v>6</v>
       </c>
       <c r="H139" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I139" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="140" ht="20" customHeight="1">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Yasmin</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
@@ -6800,7 +6800,7 @@
       </c>
       <c r="I140" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>🎓 Training Session (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6817,17 +6817,17 @@
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D141" s="5" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:15 PM</t>
         </is>
       </c>
       <c r="F141" s="5" t="inlineStr">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="I141" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -6862,7 +6862,7 @@
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>Mohammad Almohammad</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -6907,12 +6907,12 @@
       </c>
       <c r="C143" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D143" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E143" s="5" t="inlineStr">
@@ -6922,20 +6922,20 @@
       </c>
       <c r="F143" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>8h 15m</t>
         </is>
       </c>
       <c r="G143" s="7" t="n">
-        <v>8</v>
+        <v>8.25</v>
       </c>
       <c r="H143" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I143" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -6952,7 +6952,7 @@
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -6962,16 +6962,16 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G144" s="4" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
@@ -6997,7 +6997,7 @@
       </c>
       <c r="C145" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D145" s="5" t="inlineStr">
@@ -7020,12 +7020,12 @@
       </c>
       <c r="H145" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I145" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 08:00 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -7042,52 +7042,52 @@
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="147" ht="20" customHeight="1">
       <c r="A147" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B147" s="5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C147" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D147" s="5" t="inlineStr">
@@ -7122,81 +7122,81 @@
     <row r="148" ht="20" customHeight="1">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G148" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I148" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="149" ht="20" customHeight="1">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B149" s="5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Yasmin</t>
         </is>
       </c>
       <c r="D149" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F149" s="5" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G149" s="7" t="n">
-        <v>8.08</v>
+        <v>6</v>
       </c>
       <c r="H149" s="5" t="inlineStr">
         <is>
@@ -7205,7 +7205,7 @@
       </c>
       <c r="I149" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:55 AM – 04:00 PM)</t>
+          <t>🎓 Training Session (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -7222,7 +7222,7 @@
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>Mohammad Almohammad</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -7267,12 +7267,12 @@
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D151" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E151" s="5" t="inlineStr">
@@ -7282,20 +7282,20 @@
       </c>
       <c r="F151" s="5" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G151" s="7" t="n">
-        <v>8.08</v>
+        <v>8</v>
       </c>
       <c r="H151" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I151" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
@@ -7312,26 +7312,26 @@
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:55 AM</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>8h 05m</t>
         </is>
       </c>
       <c r="G152" s="4" t="n">
-        <v>8.5</v>
+        <v>8.08</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -7340,7 +7340,7 @@
       </c>
       <c r="I152" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:55 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -7357,7 +7357,7 @@
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D153" s="5" t="inlineStr">
@@ -7402,52 +7402,52 @@
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>09:00 AM</t>
+          <t>07:55 AM</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>6h 00m</t>
+          <t>8h 05m</t>
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>6</v>
+        <v>8.08</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
         <is>
-          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="155" ht="20" customHeight="1">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B155" s="5" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D155" s="5" t="inlineStr">
@@ -7457,16 +7457,16 @@
       </c>
       <c r="E155" s="5" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F155" s="5" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G155" s="7" t="n">
-        <v>5.5</v>
+        <v>8.5</v>
       </c>
       <c r="H155" s="5" t="inlineStr">
         <is>
@@ -7482,36 +7482,36 @@
     <row r="156" ht="20" customHeight="1">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>08:10 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>01:00 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>4h 50m</t>
+          <t>8h 00m</t>
         </is>
       </c>
       <c r="G156" s="4" t="n">
-        <v>4.83</v>
+        <v>8</v>
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
@@ -7527,81 +7527,81 @@
     <row r="157" ht="20" customHeight="1">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B157" s="5" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D157" s="5" t="inlineStr">
         <is>
-          <t>07:45 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F157" s="5" t="inlineStr">
         <is>
-          <t>5h 45m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G157" s="7" t="n">
-        <v>5.75</v>
+        <v>6</v>
       </c>
       <c r="H157" s="5" t="inlineStr">
         <is>
-          <t>Training / Paid</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I157" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 01:30 PM)</t>
+          <t>Daily Station Duty (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="158" ht="20" customHeight="1">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>Mohammad Almohammad</t>
+          <t>Yasmin</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>09:00 AM</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>12:30 PM</t>
+          <t>03:00 PM</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>4h 30m</t>
+          <t>6h 00m</t>
         </is>
       </c>
       <c r="G158" s="4" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
@@ -7610,7 +7610,7 @@
       </c>
       <c r="I158" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training</t>
+          <t>🎓 Training Session (09:00 AM – 03:00 PM)</t>
         </is>
       </c>
     </row>
@@ -7627,7 +7627,7 @@
       </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D159" s="5" t="inlineStr">
@@ -7637,16 +7637,16 @@
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F159" s="5" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G159" s="7" t="n">
-        <v>8.5</v>
+        <v>5.5</v>
       </c>
       <c r="H159" s="5" t="inlineStr">
         <is>
@@ -7672,26 +7672,26 @@
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>08:10 AM</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>01:00 PM</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>5h 30m</t>
+          <t>4h 50m</t>
         </is>
       </c>
       <c r="G160" s="4" t="n">
-        <v>5.5</v>
+        <v>4.83</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
@@ -7717,187 +7717,187 @@
       </c>
       <c r="C161" s="6" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D161" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>07:45 AM</t>
         </is>
       </c>
       <c r="E161" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F161" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>5h 45m</t>
         </is>
       </c>
       <c r="G161" s="7" t="n">
-        <v>9.5</v>
+        <v>5.75</v>
       </c>
       <c r="H161" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I161" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>🎓 Etihad Altéa DCS Training / HQ SERAVIA (07:45 AM – 01:30 PM)</t>
         </is>
       </c>
     </row>
     <row r="162" ht="20" customHeight="1">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>12:30 PM</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>4h 30m</t>
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="163" ht="20" customHeight="1">
       <c r="A163" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B163" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C163" s="6" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D163" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F163" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G163" s="7" t="n">
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="H163" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I163" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="164" ht="20" customHeight="1">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>07:10 AM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>8h 50m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G164" s="4" t="n">
-        <v>8.83</v>
+        <v>5.5</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Training / Paid</t>
         </is>
       </c>
       <c r="I164" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (07:10 AM – 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training</t>
         </is>
       </c>
     </row>
     <row r="165" ht="20" customHeight="1">
       <c r="A165" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B165" s="5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
-          <t>Mohammad Almohammad</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D165" s="5" t="inlineStr">
@@ -7907,16 +7907,16 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F165" s="5" t="inlineStr">
         <is>
-          <t>9h 00m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G165" s="7" t="n">
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="H165" s="5" t="inlineStr">
         <is>
@@ -7925,52 +7925,52 @@
       </c>
       <c r="I165" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="166" ht="20" customHeight="1">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Yasmin</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>06:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>05:30 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>11h 30m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G166" s="4" t="n">
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I166" s="3" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:00 AM – 04:30 PM)</t>
         </is>
       </c>
     </row>
@@ -7987,7 +7987,7 @@
       </c>
       <c r="C167" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D167" s="5" t="inlineStr">
@@ -7997,16 +7997,16 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F167" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G167" s="7" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="H167" s="5" t="inlineStr">
         <is>
@@ -8015,7 +8015,7 @@
       </c>
       <c r="I167" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>✈️ Live Morning Airport Ground Duty</t>
         </is>
       </c>
     </row>
@@ -8032,12 +8032,12 @@
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>03:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
@@ -8047,172 +8047,172 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>13h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>Dawn Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
         <is>
-          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
         </is>
       </c>
     </row>
     <row r="169" ht="20" customHeight="1">
       <c r="A169" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B169" s="5" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C169" s="6" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="D169" s="5" t="inlineStr">
         <is>
+          <t>07:10 AM</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>8h 50m</t>
+        </is>
+      </c>
+      <c r="G169" s="7" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="H169" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I169" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:10 AM – 04:00 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="20" customHeight="1">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
           <t>07:00 AM</t>
         </is>
       </c>
-      <c r="E169" s="5" t="inlineStr">
-        <is>
-          <t>03:30 PM</t>
-        </is>
-      </c>
-      <c r="F169" s="5" t="inlineStr">
-        <is>
-          <t>8h 30m</t>
-        </is>
-      </c>
-      <c r="G169" s="7" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="H169" s="5" t="inlineStr">
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G170" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
         <is>
           <t>Official Duty</t>
         </is>
       </c>
-      <c r="I169" s="6" t="inlineStr">
-        <is>
-          <t>✈️ Live Morning Airport Ground Duty</t>
-        </is>
-      </c>
-    </row>
-    <row r="170" ht="20" customHeight="1">
-      <c r="A170" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B170" s="8" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C170" s="9" t="inlineStr">
-        <is>
-          <t>Joudi Alghorani</t>
-        </is>
-      </c>
-      <c r="D170" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E170" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F170" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G170" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H170" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I170" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="I170" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 00m)</t>
         </is>
       </c>
     </row>
     <row r="171" ht="20" customHeight="1">
-      <c r="A171" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B171" s="8" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C171" s="9" t="inlineStr">
-        <is>
-          <t>Khaled</t>
-        </is>
-      </c>
-      <c r="D171" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E171" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F171" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G171" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H171" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I171" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C171" s="6" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>06:00 AM</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F171" s="5" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G171" s="7" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H171" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I171" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
         </is>
       </c>
     </row>
     <row r="172" ht="20" customHeight="1">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>Mohammad Almohammad</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -8222,115 +8222,115 @@
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>07:10 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>12h 10m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>12.17</v>
+        <v>9.5</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 07:10 PM / 12h 10m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="173" ht="20" customHeight="1">
       <c r="A173" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B173" s="5" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C173" s="6" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D173" s="5" t="inlineStr">
         <is>
-          <t>06:00 AM</t>
+          <t>03:00 AM</t>
         </is>
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t>05:30 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F173" s="5" t="inlineStr">
         <is>
-          <t>11h 30m</t>
+          <t>13h 00m</t>
         </is>
       </c>
       <c r="G173" s="7" t="n">
-        <v>11.5</v>
+        <v>13</v>
       </c>
       <c r="H173" s="5" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I173" s="6" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
         </is>
       </c>
     </row>
     <row r="174" ht="20" customHeight="1">
-      <c r="A174" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B174" s="8" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="C174" s="9" t="inlineStr">
-        <is>
-          <t>Raboushee</t>
-        </is>
-      </c>
-      <c r="D174" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E174" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F174" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G174" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H174" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I174" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>Yasmin</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G174" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:00 AM – 04:30 PM)</t>
         </is>
       </c>
     </row>
@@ -8347,7 +8347,7 @@
       </c>
       <c r="C175" s="6" t="inlineStr">
         <is>
-          <t>Rasheed Akel</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D175" s="5" t="inlineStr">
@@ -8357,42 +8357,42 @@
       </c>
       <c r="E175" s="5" t="inlineStr">
         <is>
-          <t>05:30 PM</t>
+          <t>03:30 PM</t>
         </is>
       </c>
       <c r="F175" s="5" t="inlineStr">
         <is>
-          <t>10h 30m</t>
+          <t>8h 30m</t>
         </is>
       </c>
       <c r="G175" s="7" t="n">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="H175" s="5" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Official Duty</t>
         </is>
       </c>
       <c r="I175" s="6" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 05:30 PM / 10h 30m)</t>
+          <t>✈️ Live Morning Airport Ground Duty</t>
         </is>
       </c>
     </row>
     <row r="176" ht="20" customHeight="1">
       <c r="A176" s="8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B176" s="8" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C176" s="9" t="inlineStr">
         <is>
-          <t>Hanan</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D176" s="8" t="inlineStr">
@@ -8425,119 +8425,119 @@
       </c>
     </row>
     <row r="177" ht="20" customHeight="1">
-      <c r="A177" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="B177" s="5" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C177" s="6" t="inlineStr">
-        <is>
-          <t>Joudi Alghorani</t>
-        </is>
-      </c>
-      <c r="D177" s="5" t="inlineStr">
-        <is>
-          <t>07:15 AM</t>
-        </is>
-      </c>
-      <c r="E177" s="5" t="inlineStr">
-        <is>
-          <t>04:00 PM</t>
-        </is>
-      </c>
-      <c r="F177" s="5" t="inlineStr">
-        <is>
-          <t>8h 45m</t>
-        </is>
-      </c>
-      <c r="G177" s="7" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="H177" s="5" t="inlineStr">
-        <is>
-          <t>Official Duty</t>
-        </is>
-      </c>
-      <c r="I177" s="6" t="inlineStr">
-        <is>
-          <t>✈️ Live Morning Airport Ground Duty (8h 45m)</t>
+      <c r="A177" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B177" s="8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C177" s="9" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D177" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E177" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F177" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G177" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H177" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I177" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="178" ht="20" customHeight="1">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Mohammad Almohammad</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>07:07 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>07:10 PM</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>8h 53m</t>
+          <t>12h 10m</t>
         </is>
       </c>
       <c r="G178" s="4" t="n">
-        <v>8.880000000000001</v>
+        <v>12.17</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Extended Shift</t>
         </is>
       </c>
       <c r="I178" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (07:07 AM – 04:00 PM)</t>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 07:10 PM / 12h 10m)</t>
         </is>
       </c>
     </row>
     <row r="179" ht="20" customHeight="1">
       <c r="A179" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B179" s="5" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
-          <t>Mohammad Almohammad</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D179" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>06:00 AM</t>
         </is>
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
-          <t>06:30 PM</t>
+          <t>05:30 PM</t>
         </is>
       </c>
       <c r="F179" s="5" t="inlineStr">
@@ -8555,24 +8555,24 @@
       </c>
       <c r="I179" s="6" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 06:30 PM / 11h 30m)</t>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
         </is>
       </c>
     </row>
     <row r="180" ht="20" customHeight="1">
       <c r="A180" s="8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B180" s="8" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C180" s="9" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="D180" s="8" t="inlineStr">
@@ -8600,24 +8600,24 @@
       </c>
       <c r="I180" s="9" t="inlineStr">
         <is>
-          <t>🌴 Contractual Paid Rest Day (Off Duty)</t>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="181" ht="20" customHeight="1">
       <c r="A181" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B181" s="5" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C181" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Rasheed Akel</t>
         </is>
       </c>
       <c r="D181" s="5" t="inlineStr">
@@ -8627,127 +8627,127 @@
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>05:30 PM</t>
         </is>
       </c>
       <c r="F181" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>10h 30m</t>
         </is>
       </c>
       <c r="G181" s="7" t="n">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="H181" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Extended Shift</t>
         </is>
       </c>
       <c r="I181" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:30 PM / 10h 30m)</t>
         </is>
       </c>
     </row>
     <row r="182" ht="20" customHeight="1">
       <c r="A182" s="2" t="inlineStr">
         <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>Yasmin</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>03:30 AM</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>13h 00m</t>
+        </is>
+      </c>
+      <c r="G182" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>Dawn Shift</t>
+        </is>
+      </c>
+      <c r="I182" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Early dawn flight departure handling (13h 00m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="20" customHeight="1">
+      <c r="A183" s="8" t="inlineStr">
+        <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="B183" s="8" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
       </c>
-      <c r="C182" s="3" t="inlineStr">
-        <is>
-          <t>Rasheed Akel</t>
-        </is>
-      </c>
-      <c r="D182" s="2" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="E182" s="2" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F182" s="2" t="inlineStr">
-        <is>
-          <t>5h 30m</t>
-        </is>
-      </c>
-      <c r="G182" s="4" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="H182" s="2" t="inlineStr">
-        <is>
-          <t>Afternoon Duty</t>
-        </is>
-      </c>
-      <c r="I182" s="3" t="inlineStr">
-        <is>
-          <t>✈️ Live Afternoon Station Duty (12:00 PM – 05:30 PM / 5h 30m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="183" ht="20" customHeight="1">
-      <c r="A183" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="B183" s="5" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C183" s="6" t="inlineStr">
+      <c r="C183" s="9" t="inlineStr">
         <is>
           <t>Hanan</t>
         </is>
       </c>
-      <c r="D183" s="5" t="inlineStr">
-        <is>
-          <t>03:15 AM</t>
-        </is>
-      </c>
-      <c r="E183" s="5" t="inlineStr">
-        <is>
-          <t>04:30 PM</t>
-        </is>
-      </c>
-      <c r="F183" s="5" t="inlineStr">
-        <is>
-          <t>13h 15m</t>
-        </is>
-      </c>
-      <c r="G183" s="7" t="n">
-        <v>13.25</v>
-      </c>
-      <c r="H183" s="5" t="inlineStr">
-        <is>
-          <t>Dawn Shift</t>
-        </is>
-      </c>
-      <c r="I183" s="6" t="inlineStr">
-        <is>
-          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
+      <c r="D183" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E183" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F183" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G183" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H183" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I183" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="184" ht="20" customHeight="1">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
@@ -8757,21 +8757,21 @@
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>07:20 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>04:40 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>9h 20m</t>
+          <t>8h 45m</t>
         </is>
       </c>
       <c r="G184" s="4" t="n">
-        <v>9.33</v>
+        <v>8.75</v>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
@@ -8780,19 +8780,19 @@
       </c>
       <c r="I184" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 20m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (8h 45m)</t>
         </is>
       </c>
     </row>
     <row r="185" ht="20" customHeight="1">
       <c r="A185" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B185" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C185" s="6" t="inlineStr">
@@ -8802,21 +8802,21 @@
       </c>
       <c r="D185" s="5" t="inlineStr">
         <is>
-          <t>07:20 AM</t>
+          <t>07:07 AM</t>
         </is>
       </c>
       <c r="E185" s="5" t="inlineStr">
         <is>
-          <t>04:40 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F185" s="5" t="inlineStr">
         <is>
-          <t>9h 20m</t>
+          <t>8h 53m</t>
         </is>
       </c>
       <c r="G185" s="7" t="n">
-        <v>9.33</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="H185" s="5" t="inlineStr">
         <is>
@@ -8825,109 +8825,109 @@
       </c>
       <c r="I185" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 04:40 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (07:07 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
     <row r="186" ht="20" customHeight="1">
-      <c r="A186" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="B186" s="8" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C186" s="9" t="inlineStr">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
         <is>
           <t>Mohammad Almohammad</t>
         </is>
       </c>
-      <c r="D186" s="8" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>06:30 PM</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G186" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I186" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 06:30 PM / 11h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="20" customHeight="1">
+      <c r="A187" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B187" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C187" s="9" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D187" s="8" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="E186" s="8" t="inlineStr">
+      <c r="E187" s="8" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="F186" s="8" t="inlineStr">
+      <c r="F187" s="8" t="inlineStr">
         <is>
           <t>0h 00m</t>
         </is>
       </c>
-      <c r="G186" s="10" t="n">
+      <c r="G187" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H186" s="8" t="inlineStr">
+      <c r="H187" s="8" t="inlineStr">
         <is>
           <t>Day Off</t>
         </is>
       </c>
-      <c r="I186" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Rest Day (Off Duty)</t>
-        </is>
-      </c>
-    </row>
-    <row r="187" ht="20" customHeight="1">
-      <c r="A187" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="B187" s="5" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C187" s="6" t="inlineStr">
-        <is>
-          <t>Osama Alkabbani</t>
-        </is>
-      </c>
-      <c r="D187" s="5" t="inlineStr">
-        <is>
-          <t>06:00 AM</t>
-        </is>
-      </c>
-      <c r="E187" s="5" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F187" s="5" t="inlineStr">
-        <is>
-          <t>11h 30m</t>
-        </is>
-      </c>
-      <c r="G187" s="7" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="H187" s="5" t="inlineStr">
-        <is>
-          <t>Extended Shift</t>
-        </is>
-      </c>
-      <c r="I187" s="6" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+      <c r="I187" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Contractual Paid Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="188" ht="20" customHeight="1">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
@@ -8942,16 +8942,16 @@
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>04:40 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>9h 40m</t>
+          <t>9h 30m</t>
         </is>
       </c>
       <c r="G188" s="4" t="n">
-        <v>9.67</v>
+        <v>9.5</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -8960,19 +8960,19 @@
       </c>
       <c r="I188" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 30m)</t>
         </is>
       </c>
     </row>
     <row r="189" ht="20" customHeight="1">
       <c r="A189" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B189" s="5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C189" s="6" t="inlineStr">
@@ -8982,137 +8982,137 @@
       </c>
       <c r="D189" s="5" t="inlineStr">
         <is>
-          <t>07:00 AM</t>
+          <t>12:00 PM</t>
         </is>
       </c>
       <c r="E189" s="5" t="inlineStr">
         <is>
-          <t>05:40 PM</t>
+          <t>05:30 PM</t>
         </is>
       </c>
       <c r="F189" s="5" t="inlineStr">
         <is>
-          <t>10h 40m</t>
+          <t>5h 30m</t>
         </is>
       </c>
       <c r="G189" s="7" t="n">
-        <v>10.67</v>
+        <v>5.5</v>
       </c>
       <c r="H189" s="5" t="inlineStr">
         <is>
-          <t>Extended Shift</t>
+          <t>Afternoon Duty</t>
         </is>
       </c>
       <c r="I189" s="6" t="inlineStr">
         <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+          <t>✈️ Live Afternoon Station Duty (12:00 PM – 05:30 PM / 5h 30m)</t>
         </is>
       </c>
     </row>
     <row r="190" ht="20" customHeight="1">
-      <c r="A190" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="B190" s="2" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="C190" s="3" t="inlineStr">
-        <is>
-          <t>Hanan</t>
-        </is>
-      </c>
-      <c r="D190" s="2" t="inlineStr">
-        <is>
-          <t>08:00 AM</t>
-        </is>
-      </c>
-      <c r="E190" s="2" t="inlineStr">
-        <is>
-          <t>05:00 PM</t>
-        </is>
-      </c>
-      <c r="F190" s="2" t="inlineStr">
-        <is>
-          <t>9h 00m</t>
-        </is>
-      </c>
-      <c r="G190" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="H190" s="2" t="inlineStr">
-        <is>
-          <t>Official Duty</t>
-        </is>
-      </c>
-      <c r="I190" s="3" t="inlineStr">
-        <is>
-          <t>✈️ Live Daily Ground Duty</t>
+      <c r="A190" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B190" s="8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C190" s="9" t="inlineStr">
+        <is>
+          <t>Yasmin</t>
+        </is>
+      </c>
+      <c r="D190" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E190" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F190" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G190" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H190" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I190" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="191" ht="20" customHeight="1">
       <c r="A191" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B191" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C191" s="6" t="inlineStr">
         <is>
-          <t>Joudi Alghorani</t>
+          <t>Hanan</t>
         </is>
       </c>
       <c r="D191" s="5" t="inlineStr">
         <is>
-          <t>07:30 AM</t>
+          <t>03:15 AM</t>
         </is>
       </c>
       <c r="E191" s="5" t="inlineStr">
         <is>
-          <t>04:51 PM</t>
+          <t>04:30 PM</t>
         </is>
       </c>
       <c r="F191" s="5" t="inlineStr">
         <is>
-          <t>9h 21m</t>
+          <t>13h 15m</t>
         </is>
       </c>
       <c r="G191" s="7" t="n">
-        <v>9.35</v>
+        <v>13.25</v>
       </c>
       <c r="H191" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Dawn Shift</t>
         </is>
       </c>
       <c r="I191" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Ground Duty (9h 21m)</t>
+          <t>✈️ Early dawn flight departure handling (13h 15m)</t>
         </is>
       </c>
     </row>
     <row r="192" ht="20" customHeight="1">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Joudi Alghorani</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -9122,16 +9122,16 @@
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>05:00 PM</t>
+          <t>04:40 PM</t>
         </is>
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>9h 40m</t>
+          <t>9h 20m</t>
         </is>
       </c>
       <c r="G192" s="4" t="n">
-        <v>9.67</v>
+        <v>9.33</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -9140,187 +9140,637 @@
       </c>
       <c r="I192" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 05:00 PM)</t>
+          <t>✈️ Live Morning Airport Ground Duty (9h 20m)</t>
         </is>
       </c>
     </row>
     <row r="193" ht="20" customHeight="1">
       <c r="A193" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B193" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C193" s="6" t="inlineStr">
         <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F193" s="5" t="inlineStr">
+        <is>
+          <t>9h 20m</t>
+        </is>
+      </c>
+      <c r="G193" s="7" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="H193" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I193" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 04:40 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="20" customHeight="1">
+      <c r="A194" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B194" s="8" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C194" s="9" t="inlineStr">
+        <is>
           <t>Mohammad Almohammad</t>
         </is>
       </c>
-      <c r="D193" s="5" t="inlineStr">
-        <is>
-          <t>07:00 AM</t>
-        </is>
-      </c>
-      <c r="E193" s="5" t="inlineStr">
-        <is>
-          <t>05:40 PM</t>
-        </is>
-      </c>
-      <c r="F193" s="5" t="inlineStr">
-        <is>
-          <t>10h 40m</t>
-        </is>
-      </c>
-      <c r="G193" s="7" t="n">
-        <v>10.67</v>
-      </c>
-      <c r="H193" s="5" t="inlineStr">
-        <is>
-          <t>Extended Shift</t>
-        </is>
-      </c>
-      <c r="I193" s="6" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="194" ht="20" customHeight="1">
-      <c r="A194" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="B194" s="2" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="C194" s="3" t="inlineStr">
-        <is>
-          <t>Osama Alkabbani</t>
-        </is>
-      </c>
-      <c r="D194" s="2" t="inlineStr">
-        <is>
-          <t>06:00 AM</t>
-        </is>
-      </c>
-      <c r="E194" s="2" t="inlineStr">
-        <is>
-          <t>05:30 PM</t>
-        </is>
-      </c>
-      <c r="F194" s="2" t="inlineStr">
-        <is>
-          <t>11h 30m</t>
-        </is>
-      </c>
-      <c r="G194" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="H194" s="2" t="inlineStr">
-        <is>
-          <t>Extended Shift</t>
-        </is>
-      </c>
-      <c r="I194" s="3" t="inlineStr">
-        <is>
-          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+      <c r="D194" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E194" s="8" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F194" s="8" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G194" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H194" s="8" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I194" s="9" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
         </is>
       </c>
     </row>
     <row r="195" ht="20" customHeight="1">
       <c r="A195" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B195" s="5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C195" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="D195" s="5" t="inlineStr">
         <is>
-          <t>07:30 AM</t>
+          <t>06:00 AM</t>
         </is>
       </c>
       <c r="E195" s="5" t="inlineStr">
         <is>
-          <t>05:00 PM</t>
+          <t>05:30 PM</t>
         </is>
       </c>
       <c r="F195" s="5" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>11h 30m</t>
         </is>
       </c>
       <c r="G195" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="H195" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Extended Shift</t>
         </is>
       </c>
       <c r="I195" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Ground Duty (9h 30m)</t>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
         </is>
       </c>
     </row>
     <row r="196" ht="20" customHeight="1">
       <c r="A196" s="2" t="inlineStr">
         <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>04:40 PM</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>9h 40m</t>
+        </is>
+      </c>
+      <c r="G196" s="4" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I196" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (9h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="20" customHeight="1">
+      <c r="A197" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B197" s="5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C197" s="6" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D197" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E197" s="5" t="inlineStr">
+        <is>
+          <t>05:40 PM</t>
+        </is>
+      </c>
+      <c r="F197" s="5" t="inlineStr">
+        <is>
+          <t>10h 40m</t>
+        </is>
+      </c>
+      <c r="G197" s="7" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="H197" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I197" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="20" customHeight="1">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>Yasmin</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>04:00 AM</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>12h 30m</t>
+        </is>
+      </c>
+      <c r="G198" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>Dawn Shift</t>
+        </is>
+      </c>
+      <c r="I198" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Early dawn flight departure handling (12h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="20" customHeight="1">
+      <c r="A199" s="5" t="inlineStr">
+        <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B196" s="2" t="inlineStr">
+      <c r="B199" s="5" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C196" s="3" t="inlineStr">
+      <c r="C199" s="6" t="inlineStr">
+        <is>
+          <t>Hanan</t>
+        </is>
+      </c>
+      <c r="D199" s="5" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E199" s="5" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F199" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G199" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H199" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I199" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="20" customHeight="1">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>Joudi Alghorani</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>07:30 AM</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>04:51 PM</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>9h 21m</t>
+        </is>
+      </c>
+      <c r="G200" s="4" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I200" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (9h 21m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="20" customHeight="1">
+      <c r="A201" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B201" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C201" s="6" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D201" s="5" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="E201" s="5" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F201" s="5" t="inlineStr">
+        <is>
+          <t>9h 40m</t>
+        </is>
+      </c>
+      <c r="G201" s="7" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="H201" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I201" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 05:00 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="20" customHeight="1">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>05:40 PM</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>10h 40m</t>
+        </is>
+      </c>
+      <c r="G202" s="4" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I202" s="3" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 05:40 PM / 10h 40m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="20" customHeight="1">
+      <c r="A203" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B203" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C203" s="6" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D203" s="5" t="inlineStr">
+        <is>
+          <t>06:00 AM</t>
+        </is>
+      </c>
+      <c r="E203" s="5" t="inlineStr">
+        <is>
+          <t>05:30 PM</t>
+        </is>
+      </c>
+      <c r="F203" s="5" t="inlineStr">
+        <is>
+          <t>11h 30m</t>
+        </is>
+      </c>
+      <c r="G203" s="7" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H203" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I203" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (06:00 AM – 05:30 PM / 11h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="20" customHeight="1">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>Raboushee</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>07:30 AM</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>9h 30m</t>
+        </is>
+      </c>
+      <c r="G204" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I204" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (9h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="20" customHeight="1">
+      <c r="A205" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B205" s="5" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C205" s="6" t="inlineStr">
         <is>
           <t>Rasheed Akel</t>
         </is>
       </c>
-      <c r="D196" s="2" t="inlineStr">
+      <c r="D205" s="5" t="inlineStr">
         <is>
           <t>07:00 AM</t>
         </is>
       </c>
-      <c r="E196" s="2" t="inlineStr">
+      <c r="E205" s="5" t="inlineStr">
         <is>
           <t>05:00 PM</t>
         </is>
       </c>
-      <c r="F196" s="2" t="inlineStr">
+      <c r="F205" s="5" t="inlineStr">
         <is>
           <t>10h 00m</t>
         </is>
       </c>
-      <c r="G196" s="4" t="n">
+      <c r="G205" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="H196" s="2" t="inlineStr">
+      <c r="H205" s="5" t="inlineStr">
         <is>
           <t>Extended Shift</t>
         </is>
       </c>
-      <c r="I196" s="3" t="inlineStr">
+      <c r="I205" s="6" t="inlineStr">
         <is>
           <t>⚡ Live Extended Station Duty (07:00 AM – 05:00 PM / 10h 00m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="20" customHeight="1">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>Yasmin</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>05:00 PM</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G206" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I206" s="3" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Ground Duty (08:00 AM – 05:00 PM)</t>
         </is>
       </c>
     </row>
@@ -9864,7 +10314,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>06:30 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -9874,20 +10324,20 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>9h 30m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Standardized</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Standardized 23rd shift: 06:30 AM – 04:00 PM (9.5h)</t>
+          <t>Standard morning bus shift (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -10359,7 +10809,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -10369,11 +10819,11 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
@@ -10382,7 +10832,7 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Standard daytime shift</t>
+          <t>Standard morning bus shift (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -10854,7 +11304,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:00 AM</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -10864,11 +11314,11 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 00m</t>
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -10877,7 +11327,7 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Standard daytime shift</t>
+          <t>Standard morning bus shift (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -11332,47 +11782,47 @@
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>Yasmin</t>
         </is>
       </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G45" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I45" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled weekly day off</t>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Standard morning bus shift (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -11867,7 +12317,7 @@
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>Morning flight shift</t>
+          <t>Standard morning bus shift (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -12362,7 +12812,7 @@
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>Morning flight shift</t>
+          <t>Standard morning bus shift (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -12857,7 +13307,7 @@
       </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>Morning flight shift (4:00 PM return)</t>
+          <t>Standard morning bus shift (07:00 AM – 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -13504,20 +13954,20 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Osama Alkabbani</t>
+          <t>Yasmin</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
         <v>72</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>174</v>
+        <v>175.25</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>246</v>
+        <v>247.25</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -13526,20 +13976,20 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Khaled</t>
+          <t>Osama Alkabbani</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>172.68</v>
+        <v>174</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>243.68</v>
+        <v>246</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -13548,20 +13998,20 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Khaled</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>69.33</v>
+        <v>71</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>169.67</v>
+        <v>172.68</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>239</v>
+        <v>243.68</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -13570,20 +14020,20 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>66.67</v>
+        <v>69.33</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>107.09</v>
+        <v>169.67</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>173.76</v>
+        <v>239</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -13592,20 +14042,20 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Yasmin</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>61.5</v>
+        <v>66.67</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>69.72</v>
+        <v>107.09</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>131.22</v>
+        <v>173.76</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Adjust Omar shift times (+40m in/out) Oct 5-21 and log Oct 22 check-in at 07:15 AM
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -39,7 +39,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +62,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -121,6 +127,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -488,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I212"/>
+  <dimension ref="A1:I213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2727,21 +2742,21 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:20 AM</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:40 PM</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 20m</t>
         </is>
       </c>
       <c r="G50" s="4" t="n">
-        <v>8</v>
+        <v>9.33</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -3222,21 +3237,21 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:20 AM</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>04:05 PM</t>
+          <t>04:45 PM</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>9h 25m</t>
         </is>
       </c>
       <c r="G61" s="7" t="n">
-        <v>8.08</v>
+        <v>9.42</v>
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
@@ -3717,21 +3732,21 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>7h 25m</t>
+          <t>8h 45m</t>
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>7.42</v>
+        <v>8.75</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3740,7 +3755,7 @@
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Airport Ground Station Duty (Logged in 07:55 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Airport Ground Station Duty (Logged in 07:15 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -4212,21 +4227,21 @@
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>07:50 AM</t>
+          <t>07:10 AM</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>7h 30m</t>
+          <t>8h 50m</t>
         </is>
       </c>
       <c r="G83" s="7" t="n">
-        <v>7.5</v>
+        <v>8.83</v>
       </c>
       <c r="H83" s="5" t="inlineStr">
         <is>
@@ -4235,7 +4250,7 @@
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:50 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Daily Duty (Logged in 07:10 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -4707,21 +4722,21 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>07:50 AM</t>
+          <t>07:10 AM</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>05:13 PM</t>
+          <t>05:53 PM</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>9h 23m</t>
+          <t>10h 43m</t>
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>9.380000000000001</v>
+        <v>10.72</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -4730,7 +4745,7 @@
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:50 AM / Logged out 05:13 PM)</t>
+          <t>✈️ Live Daily Duty (Logged in 07:10 AM / Logged out 05:53 PM)</t>
         </is>
       </c>
     </row>
@@ -5202,21 +5217,21 @@
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>07:47 AM</t>
+          <t>07:07 AM</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>03:35 PM</t>
+          <t>04:15 PM</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>7h 48m</t>
+          <t>9h 08m</t>
         </is>
       </c>
       <c r="G105" s="7" t="n">
-        <v>7.8</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="H105" s="5" t="inlineStr">
         <is>
@@ -5225,7 +5240,7 @@
       </c>
       <c r="I105" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:47 AM / Logged out 03:35 PM)</t>
+          <t>✈️ Live Daily Duty (Logged in 07:07 AM / Logged out 04:15 PM)</t>
         </is>
       </c>
     </row>
@@ -6192,21 +6207,21 @@
       </c>
       <c r="D127" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>05:05 PM</t>
+          <t>05:45 PM</t>
         </is>
       </c>
       <c r="F127" s="5" t="inlineStr">
         <is>
-          <t>9h 10m</t>
+          <t>10h 30m</t>
         </is>
       </c>
       <c r="G127" s="7" t="n">
-        <v>9.17</v>
+        <v>10.5</v>
       </c>
       <c r="H127" s="5" t="inlineStr">
         <is>
@@ -6215,7 +6230,7 @@
       </c>
       <c r="I127" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:55 AM / Logged out 05:05 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:15 AM / Logged out 05:45 PM)</t>
         </is>
       </c>
     </row>
@@ -6597,21 +6612,21 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:20 AM</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>04:30 PM</t>
+          <t>05:10 PM</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>8h 30m</t>
+          <t>9h 50m</t>
         </is>
       </c>
       <c r="G136" s="4" t="n">
-        <v>8.5</v>
+        <v>9.83</v>
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
@@ -6620,7 +6635,7 @@
       </c>
       <c r="I136" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 08:00 AM / Logged out 04:30 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:20 AM / Logged out 05:10 PM)</t>
         </is>
       </c>
     </row>
@@ -7002,21 +7017,21 @@
       </c>
       <c r="D145" s="5" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:20 AM</t>
         </is>
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:40 PM</t>
         </is>
       </c>
       <c r="F145" s="5" t="inlineStr">
         <is>
-          <t>8h 00m</t>
+          <t>9h 20m</t>
         </is>
       </c>
       <c r="G145" s="7" t="n">
-        <v>8</v>
+        <v>9.33</v>
       </c>
       <c r="H145" s="5" t="inlineStr">
         <is>
@@ -7025,7 +7040,7 @@
       </c>
       <c r="I145" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 08:00 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:20 AM / Logged out 04:40 PM)</t>
         </is>
       </c>
     </row>
@@ -7407,21 +7422,21 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>04:00 PM</t>
+          <t>04:40 PM</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>8h 05m</t>
+          <t>9h 25m</t>
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>8.08</v>
+        <v>9.42</v>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
@@ -7430,7 +7445,7 @@
       </c>
       <c r="I154" s="3" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:55 AM / Logged out 04:00 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:15 AM / Logged out 04:40 PM)</t>
         </is>
       </c>
     </row>
@@ -7812,21 +7827,21 @@
       </c>
       <c r="D163" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>12:30 PM</t>
+          <t>01:10 PM</t>
         </is>
       </c>
       <c r="F163" s="5" t="inlineStr">
         <is>
-          <t>4h 35m</t>
+          <t>5h 55m</t>
         </is>
       </c>
       <c r="G163" s="7" t="n">
-        <v>4.58</v>
+        <v>5.92</v>
       </c>
       <c r="H163" s="5" t="inlineStr">
         <is>
@@ -7835,7 +7850,7 @@
       </c>
       <c r="I163" s="6" t="inlineStr">
         <is>
-          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:55 AM / Logged out 12:30 PM)</t>
+          <t>🎓 Etihad Airways Altéa DCS System Training (Logged in 07:15 AM / Logged out 01:10 PM)</t>
         </is>
       </c>
     </row>
@@ -8217,21 +8232,21 @@
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>07:20 AM</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>03:37 PM</t>
+          <t>04:17 PM</t>
         </is>
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>7h 37m</t>
+          <t>8h 57m</t>
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>7.62</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -8240,7 +8255,7 @@
       </c>
       <c r="I172" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 08:00 AM / Logged out 03:37 PM | Free Zone Bus: Arr 07:03 PM, Dep 07:23 PM)</t>
+          <t>✈️ Live Daily Duty (Logged in 07:20 AM / Logged out 04:17 PM | Free Zone Bus: Arr 07:03 PM, Dep 07:23 PM)</t>
         </is>
       </c>
     </row>
@@ -9027,21 +9042,21 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>03:20 PM</t>
+          <t>04:00 PM</t>
         </is>
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>7h 25m</t>
+          <t>8h 45m</t>
         </is>
       </c>
       <c r="G190" s="4" t="n">
-        <v>7.42</v>
+        <v>8.75</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -9050,7 +9065,7 @@
       </c>
       <c r="I190" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:55 AM / Logged out 03:20 PM)</t>
+          <t>✈️ Live Daily Duty (Logged in 07:15 AM / Logged out 04:00 PM)</t>
         </is>
       </c>
     </row>
@@ -9432,21 +9447,21 @@
       </c>
       <c r="D199" s="5" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
         <is>
-          <t>06:24 PM</t>
+          <t>07:04 PM</t>
         </is>
       </c>
       <c r="F199" s="5" t="inlineStr">
         <is>
-          <t>10h 29m</t>
+          <t>11h 49m</t>
         </is>
       </c>
       <c r="G199" s="7" t="n">
-        <v>10.48</v>
+        <v>11.82</v>
       </c>
       <c r="H199" s="5" t="inlineStr">
         <is>
@@ -9455,7 +9470,7 @@
       </c>
       <c r="I199" s="6" t="inlineStr">
         <is>
-          <t>⚡ Extended Shift / Overtime (Logged in 07:55 AM / Logged out 06:24 PM)</t>
+          <t>⚡ Extended Shift / Overtime (Logged in 07:15 AM / Logged out 07:04 PM)</t>
         </is>
       </c>
     </row>
@@ -9837,21 +9852,21 @@
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>07:55 AM</t>
+          <t>07:15 AM</t>
         </is>
       </c>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>04:20 PM</t>
+          <t>05:00 PM</t>
         </is>
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>8h 25m</t>
+          <t>9h 45m</t>
         </is>
       </c>
       <c r="G208" s="4" t="n">
-        <v>8.42</v>
+        <v>9.75</v>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
@@ -9860,7 +9875,7 @@
       </c>
       <c r="I208" s="3" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:55 AM / Logged out 04:20 PM)</t>
+          <t>✈️ Live Daily Duty (Logged in 07:15 AM / Logged out 05:00 PM)</t>
         </is>
       </c>
     </row>
@@ -10041,6 +10056,51 @@
       <c r="I212" s="3" t="inlineStr">
         <is>
           <t>✈️ Live Daily Ground Duty (08:00 AM – 05:00 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="20" customHeight="1">
+      <c r="A213" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B213" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C213" s="12" t="inlineStr">
+        <is>
+          <t>Omar Elnemr</t>
+        </is>
+      </c>
+      <c r="D213" s="11" t="inlineStr">
+        <is>
+          <t>07:15 AM</t>
+        </is>
+      </c>
+      <c r="E213" s="11" t="inlineStr">
+        <is>
+          <t>To Be Updated</t>
+        </is>
+      </c>
+      <c r="F213" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G213" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H213" s="11" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I213" s="12" t="inlineStr">
+        <is>
+          <t>✈️ Live Daily Duty (Logged in 07:15 AM / Awaiting Checkout)</t>
         </is>
       </c>
     </row>
@@ -14319,10 +14379,10 @@
         <v>66.67</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>147.45</v>
+        <v>167.45</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>214.12</v>
+        <v>234.12</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>26</v>

</xml_diff>

<commit_message>
Update Omar Oct 2 to 9.0h Paid Administrative Standby (airport pass delay)
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -1240,47 +1240,47 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Omar Elnemr</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>0h 00m</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>🌴 Scheduled Team Rest Day (Contractual 1 Day Off in 7-day cycle)</t>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>04:00 PM</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>🏢 Paid Administrative Standby (Damascus Airport Pass Delay - Company Paid)</t>
         </is>
       </c>
     </row>
@@ -14350,17 +14350,17 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Raboushee</t>
+          <t>Omar Elnemr</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>69.33</v>
+        <v>66.67</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>169.67</v>
+        <v>176.45</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>239</v>
+        <v>243.12</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>27</v>
@@ -14372,20 +14372,20 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Omar Elnemr</t>
+          <t>Raboushee</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>66.67</v>
+        <v>69.33</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>167.45</v>
+        <v>169.67</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>234.12</v>
+        <v>239</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Complete Omar Oct 22 shift: 07:15 AM - 06:40 PM (11h 25m / Overtime)
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -10082,16 +10082,16 @@
       </c>
       <c r="E213" s="11" t="inlineStr">
         <is>
-          <t>To Be Updated</t>
+          <t>06:40 PM</t>
         </is>
       </c>
       <c r="F213" s="11" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>11h 25m</t>
         </is>
       </c>
       <c r="G213" s="13" t="n">
-        <v>0</v>
+        <v>11.42</v>
       </c>
       <c r="H213" s="11" t="inlineStr">
         <is>
@@ -10100,7 +10100,7 @@
       </c>
       <c r="I213" s="12" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Duty (Logged in 07:15 AM / Awaiting Checkout)</t>
+          <t>⚡ Extended Shift / Overtime (Logged in 07:15 AM / Logged out 06:40 PM)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete Omar Oct 23 shift: 07:20 AM - 07:30 PM (12h 10m / Overtime)
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I213"/>
+  <dimension ref="A1:I214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10101,6 +10101,51 @@
       <c r="I213" s="12" t="inlineStr">
         <is>
           <t>⚡ Extended Shift / Overtime (Logged in 07:15 AM / Logged out 06:40 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B214" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C214" s="6" t="inlineStr">
+        <is>
+          <t>Omar Elnemr</t>
+        </is>
+      </c>
+      <c r="D214" s="5" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="E214" s="5" t="inlineStr">
+        <is>
+          <t>07:30 PM</t>
+        </is>
+      </c>
+      <c r="F214" s="5" t="inlineStr">
+        <is>
+          <t>12h 10m</t>
+        </is>
+      </c>
+      <c r="G214" s="7" t="n">
+        <v>12.17</v>
+      </c>
+      <c r="H214" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I214" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Extended Shift / Overtime (Logged in 07:20 AM / Logged out 07:30 PM)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Omar Oct 24 shift logout to 03:40 PM (8h 16m)
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -10172,16 +10172,16 @@
       </c>
       <c r="E215" s="5" t="inlineStr">
         <is>
-          <t>03:00 PM</t>
+          <t>03:40 PM</t>
         </is>
       </c>
       <c r="F215" s="5" t="inlineStr">
         <is>
-          <t>7h 36m</t>
+          <t>8h 16m</t>
         </is>
       </c>
       <c r="G215" s="7" t="n">
-        <v>7.6</v>
+        <v>8.27</v>
       </c>
       <c r="H215" s="5" t="inlineStr">
         <is>
@@ -10190,7 +10190,7 @@
       </c>
       <c r="I215" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Daily Ground Duty (Logged in 07:24 AM / Logged out 03:00 PM)</t>
+          <t>✈️ Live Daily Ground Duty (Logged in 07:24 AM / Logged out 03:40 PM)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Mohammad Almohammad attendance: Oct 22 (11h), Oct 23 (11h), Oct 24 (9h 40m)
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I215"/>
+  <dimension ref="A1:I218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10191,6 +10191,141 @@
       <c r="I215" s="6" t="inlineStr">
         <is>
           <t>✈️ Live Daily Ground Duty (Logged in 07:24 AM / Logged out 03:40 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B216" s="5" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C216" s="6" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D216" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E216" s="5" t="inlineStr">
+        <is>
+          <t>06:00 PM</t>
+        </is>
+      </c>
+      <c r="F216" s="5" t="inlineStr">
+        <is>
+          <t>11h 00m</t>
+        </is>
+      </c>
+      <c r="G216" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="H216" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I216" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 06:00 PM / 11h 00m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B217" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C217" s="6" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D217" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E217" s="5" t="inlineStr">
+        <is>
+          <t>06:00 PM</t>
+        </is>
+      </c>
+      <c r="F217" s="5" t="inlineStr">
+        <is>
+          <t>11h 00m</t>
+        </is>
+      </c>
+      <c r="G217" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="H217" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I217" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 06:00 PM / 11h 00m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B218" s="5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C218" s="6" t="inlineStr">
+        <is>
+          <t>Mohammad Almohammad</t>
+        </is>
+      </c>
+      <c r="D218" s="5" t="inlineStr">
+        <is>
+          <t>08:00 AM</t>
+        </is>
+      </c>
+      <c r="E218" s="5" t="inlineStr">
+        <is>
+          <t>05:40 PM</t>
+        </is>
+      </c>
+      <c r="F218" s="5" t="inlineStr">
+        <is>
+          <t>9h 40m</t>
+        </is>
+      </c>
+      <c r="G218" s="7" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="H218" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I218" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (08:00 AM – 05:40 PM / 9h 40m)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Khaled Malas attendance (Oct 22-24)
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I230"/>
+  <dimension ref="A1:I233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10866,6 +10866,141 @@
       <c r="I230" s="6" t="inlineStr">
         <is>
           <t>✈️ Live Morning Airport Ground Duty (07:30 AM – 03:45 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B231" s="5" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C231" s="6" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D231" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E231" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F231" s="5" t="inlineStr">
+        <is>
+          <t>0h 00m</t>
+        </is>
+      </c>
+      <c r="G231" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H231" s="5" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="I231" s="6" t="inlineStr">
+        <is>
+          <t>🌴 Scheduled Rest Day (Off Duty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B232" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C232" s="6" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D232" s="5" t="inlineStr">
+        <is>
+          <t>07:30 AM</t>
+        </is>
+      </c>
+      <c r="E232" s="5" t="inlineStr">
+        <is>
+          <t>06:00 PM</t>
+        </is>
+      </c>
+      <c r="F232" s="5" t="inlineStr">
+        <is>
+          <t>10h 30m</t>
+        </is>
+      </c>
+      <c r="G232" s="7" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H232" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I232" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:30 AM – 06:00 PM / 10h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B233" s="5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C233" s="6" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D233" s="5" t="inlineStr">
+        <is>
+          <t>07:20 AM</t>
+        </is>
+      </c>
+      <c r="E233" s="5" t="inlineStr">
+        <is>
+          <t>03:45 PM</t>
+        </is>
+      </c>
+      <c r="F233" s="5" t="inlineStr">
+        <is>
+          <t>8h 25m</t>
+        </is>
+      </c>
+      <c r="G233" s="7" t="n">
+        <v>8.42</v>
+      </c>
+      <c r="H233" s="5" t="inlineStr">
+        <is>
+          <t>Official Duty</t>
+        </is>
+      </c>
+      <c r="I233" s="6" t="inlineStr">
+        <is>
+          <t>✈️ Live Morning Airport Ground Duty (07:20 AM – 03:45 PM)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Mohammad Almohammad Oct 24 logout to 18:20 (10h 20m)
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -10307,25 +10307,25 @@
       </c>
       <c r="E218" s="5" t="inlineStr">
         <is>
-          <t>05:40 PM</t>
+          <t>06:20 PM</t>
         </is>
       </c>
       <c r="F218" s="5" t="inlineStr">
         <is>
-          <t>9h 40m</t>
+          <t>10h 20m</t>
         </is>
       </c>
       <c r="G218" s="7" t="n">
-        <v>9.67</v>
+        <v>10.33</v>
       </c>
       <c r="H218" s="5" t="inlineStr">
         <is>
-          <t>Official Duty</t>
+          <t>Extended Shift</t>
         </is>
       </c>
       <c r="I218" s="6" t="inlineStr">
         <is>
-          <t>✈️ Live Morning Airport Ground Duty (08:00 AM – 05:40 PM / 9h 40m)</t>
+          <t>⚡ Live Extended Station Duty (08:00 AM – 06:20 PM / 10h 20m)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Rasheed Akel Oct 25 shift: 07:00 AM - 07:20 PM (12h 20m)
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I219"/>
+  <dimension ref="A1:I220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10371,6 +10371,51 @@
       <c r="I219" s="6" t="inlineStr">
         <is>
           <t>✈️ Live Airport Ground Station Night Duty (Logged in 08:00 PM / Logged out 03:10 AM next day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B220" s="5" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C220" s="6" t="inlineStr">
+        <is>
+          <t>Rasheed Akel</t>
+        </is>
+      </c>
+      <c r="D220" s="5" t="inlineStr">
+        <is>
+          <t>07:00 AM</t>
+        </is>
+      </c>
+      <c r="E220" s="5" t="inlineStr">
+        <is>
+          <t>07:20 PM</t>
+        </is>
+      </c>
+      <c r="F220" s="5" t="inlineStr">
+        <is>
+          <t>12h 20m</t>
+        </is>
+      </c>
+      <c r="G220" s="7" t="n">
+        <v>12.33</v>
+      </c>
+      <c r="H220" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I220" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (07:00 AM – 07:20 PM / 12h 20m)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Osama Alkabbani Oct 26 shift: 05:30 AM - 07:00 PM (13h 30m)
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I222"/>
+  <dimension ref="A1:I223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10506,6 +10506,51 @@
       <c r="I222" s="6" t="inlineStr">
         <is>
           <t>⚡ Live Extended Station Duty (07:00 AM – 07:06 PM / 12h 06m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B223" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C223" s="6" t="inlineStr">
+        <is>
+          <t>Osama Alkabbani</t>
+        </is>
+      </c>
+      <c r="D223" s="5" t="inlineStr">
+        <is>
+          <t>05:30 AM</t>
+        </is>
+      </c>
+      <c r="E223" s="5" t="inlineStr">
+        <is>
+          <t>07:00 PM</t>
+        </is>
+      </c>
+      <c r="F223" s="5" t="inlineStr">
+        <is>
+          <t>13h 30m</t>
+        </is>
+      </c>
+      <c r="G223" s="7" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H223" s="5" t="inlineStr">
+        <is>
+          <t>Extended Shift</t>
+        </is>
+      </c>
+      <c r="I223" s="6" t="inlineStr">
+        <is>
+          <t>⚡ Live Extended Station Duty (05:30 AM – 07:00 PM / 13h 30m)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Generate HR single-day file for 2026-10-26 with flight cancellation paid standby
</commit_message>
<xml_diff>
--- a/attendance_master_2026.xlsx
+++ b/attendance_master_2026.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I223"/>
+  <dimension ref="A1:I226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10551,6 +10551,141 @@
       <c r="I223" s="6" t="inlineStr">
         <is>
           <t>⚡ Live Extended Station Duty (05:30 AM – 07:00 PM / 13h 30m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B224" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C224" s="6" t="inlineStr">
+        <is>
+          <t>Omar Elnemr</t>
+        </is>
+      </c>
+      <c r="D224" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E224" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F224" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G224" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H224" s="5" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="I224" s="6" t="inlineStr">
+        <is>
+          <t>🏢 Company Paid Standby (Flight Cancelled - Station Standby)</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B225" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C225" s="6" t="inlineStr">
+        <is>
+          <t>Khaled</t>
+        </is>
+      </c>
+      <c r="D225" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E225" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F225" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G225" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H225" s="5" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="I225" s="6" t="inlineStr">
+        <is>
+          <t>🏢 Company Paid Standby (Flight Cancelled - Station Standby)</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B226" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C226" s="6" t="inlineStr">
+        <is>
+          <t>Yasmin</t>
+        </is>
+      </c>
+      <c r="D226" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E226" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F226" s="5" t="inlineStr">
+        <is>
+          <t>9h 00m</t>
+        </is>
+      </c>
+      <c r="G226" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H226" s="5" t="inlineStr">
+        <is>
+          <t>Paid Standby</t>
+        </is>
+      </c>
+      <c r="I226" s="6" t="inlineStr">
+        <is>
+          <t>🏢 Company Paid Standby (Flight Cancelled - Station Standby)</t>
         </is>
       </c>
     </row>

</xml_diff>